<commit_message>
Fixed GL Account Errors
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harih\OneDrive\Documents\UiPath\Invoices\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB09485-084A-4881-BDCD-EAE66C2090D5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F5C0FB8-2C29-4391-A3C3-2028BD8C83A6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,13 @@
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" r:id="rId3"/>
-    <sheet name="TCP DEL" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="445">
   <si>
     <t>Name</t>
   </si>
@@ -483,15 +482,6 @@
     <t>TimeOut_Logout</t>
   </si>
   <si>
-    <t>Treasury Confirmation Process - User Input Form</t>
-  </si>
-  <si>
-    <t>ColName_Status</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
     <t>SheetName_InputFile</t>
   </si>
   <si>
@@ -501,48 +491,12 @@
     <t>Validating Input file for invalid data</t>
   </si>
   <si>
-    <t>Accomplished Date</t>
-  </si>
-  <si>
-    <t>ColName_AccomplishedDate</t>
-  </si>
-  <si>
-    <t>Payment Instruction</t>
-  </si>
-  <si>
-    <t>ColName_PaymentInstruction</t>
-  </si>
-  <si>
-    <t>Accomplished Date - Invalid Date Format</t>
-  </si>
-  <si>
-    <t>BotStatus_AccomplishedDate_InvalidDateFormat</t>
-  </si>
-  <si>
     <t>BotStatus_PaymentInstruction_InvalidData</t>
   </si>
   <si>
     <t>PaymentInstruction - Invalid Data</t>
   </si>
   <si>
-    <t>Range Sequence</t>
-  </si>
-  <si>
-    <t>From</t>
-  </si>
-  <si>
-    <t>To</t>
-  </si>
-  <si>
-    <t>ColName_RangeSequence</t>
-  </si>
-  <si>
-    <t>ColName_From</t>
-  </si>
-  <si>
-    <t>ColName_To</t>
-  </si>
-  <si>
     <t>BotStatus_RangeSequence_InvalidData</t>
   </si>
   <si>
@@ -591,111 +545,21 @@
     <t>DOL Federal Administrator</t>
   </si>
   <si>
-    <t>Log_NavigateToTreasuryConfirmation</t>
-  </si>
-  <si>
-    <t>Navigating to Treasury Confirmation</t>
-  </si>
-  <si>
-    <t>Log_NavigateToTreasuryConfirmationSuccess</t>
-  </si>
-  <si>
-    <t>Navigating to Treasury Confirmation - Success</t>
-  </si>
-  <si>
     <t>SE_ErrMsg_FederalAdministratorNotDisplayed</t>
   </si>
   <si>
     <t>DOL Federal Administrator Not Displayed</t>
   </si>
   <si>
-    <t>SE_ErrMsg_TreasuryConfirmationNotDisplayed</t>
-  </si>
-  <si>
-    <t>Treasury Confirmation Not Displayed</t>
-  </si>
-  <si>
-    <t>ColName_ProcessType</t>
-  </si>
-  <si>
-    <t>ProcessType</t>
-  </si>
-  <si>
-    <t>Transaction Complete</t>
-  </si>
-  <si>
-    <t>ColName_RequestNumber</t>
-  </si>
-  <si>
-    <t>Request Number</t>
-  </si>
-  <si>
-    <t>ColName_ReferenceAssignedbyAdmin</t>
-  </si>
-  <si>
-    <t>Reference Assigned by Admin</t>
-  </si>
-  <si>
-    <t>Date Sent to Treasury</t>
-  </si>
-  <si>
-    <t>ColName_DateSentToTreasury</t>
-  </si>
-  <si>
-    <t>BotStatus_DateSentToTreasury_InvalidDateFormat</t>
-  </si>
-  <si>
-    <t>Date Sent To Treasury - Invalid Date Format</t>
-  </si>
-  <si>
-    <t>Treasury Confirmation - Report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attached is the bot generated Treasury Confirmation Report. </t>
-  </si>
-  <si>
     <t>Treasury Confirmation - Error Occurred</t>
   </si>
   <si>
-    <t>MaxNumOfValidationLoops</t>
-  </si>
-  <si>
-    <t>Number</t>
-  </si>
-  <si>
     <t>Status_InProgress</t>
   </si>
   <si>
     <t>In Progress - Check Concurrent Manager</t>
   </si>
   <si>
-    <t>Confirm</t>
-  </si>
-  <si>
-    <t>BackOut</t>
-  </si>
-  <si>
-    <t>ProcessType_Confirm</t>
-  </si>
-  <si>
-    <t>ProcessType_BackOut</t>
-  </si>
-  <si>
-    <t>BRE_InvalidPaymentInstructon</t>
-  </si>
-  <si>
-    <t>Entered 'PaymentInstruction' is invalid</t>
-  </si>
-  <si>
-    <t>Log_PaymentCount</t>
-  </si>
-  <si>
-    <t>Account Entries need to be created</t>
-  </si>
-  <si>
-    <t>BRE_AccountEntryError</t>
-  </si>
-  <si>
     <t>Log_RequestNumber</t>
   </si>
   <si>
@@ -786,45 +650,9 @@
     <t>Log_SingleRangeEntrySuccess</t>
   </si>
   <si>
-    <t>Log_ReOpenTreasuryConfirmation</t>
-  </si>
-  <si>
-    <t>ReOpening Treasury Confirmation</t>
-  </si>
-  <si>
-    <t>Log_ReOpenTreasuryConfirmationSuccess</t>
-  </si>
-  <si>
-    <t>ReOpening Treasury Confirmation - Success</t>
-  </si>
-  <si>
-    <t>BRE_FieldsNotMatch</t>
-  </si>
-  <si>
-    <t>BRE_InvalidBackOut</t>
-  </si>
-  <si>
-    <t>Invalid Back Out</t>
-  </si>
-  <si>
-    <t>Payment Instruction Fields did not match</t>
-  </si>
-  <si>
     <t>TimeOut_BackOutRequestNumberNote</t>
   </si>
   <si>
-    <t>ViewLog_StartIndex</t>
-  </si>
-  <si>
-    <t>ViewLog_EndIndex</t>
-  </si>
-  <si>
-    <t>Start of log messages from FND_FILE</t>
-  </si>
-  <si>
-    <t>End of log messages from FND_FILE</t>
-  </si>
-  <si>
     <t>Log Message(s) for Unconfirmed Payment Instruction -</t>
   </si>
   <si>
@@ -853,15 +681,6 @@
   </si>
   <si>
     <t>Unconfirmed</t>
-  </si>
-  <si>
-    <t>AdjustRowHeight</t>
-  </si>
-  <si>
-    <t>in number</t>
-  </si>
-  <si>
-    <t>gmahesh2789@gmail.com; hariharangouri@gmail.com</t>
   </si>
   <si>
     <t>gmahesh2789@gmail.com; hariharangouri@gmail.com; sunil.melam@gmail.com</t>
@@ -1992,7 +1811,7 @@
         <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>304</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -2042,7 +1861,7 @@
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>42</v>
@@ -2054,10 +1873,10 @@
     </row>
     <row r="12" spans="1:26" ht="14.5">
       <c r="A12" s="2" t="s">
-        <v>386</v>
+        <v>326</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>350</v>
+        <v>290</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="15" customHeight="1">
@@ -2088,279 +1907,279 @@
     </row>
     <row r="16" spans="1:26" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>443</v>
+        <v>383</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>444</v>
+        <v>384</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>305</v>
+        <v>245</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>306</v>
+        <v>246</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>328</v>
+        <v>268</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>307</v>
+        <v>247</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>329</v>
+        <v>269</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>308</v>
+        <v>248</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>330</v>
+        <v>270</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>309</v>
+        <v>249</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>359</v>
+        <v>299</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>310</v>
+        <v>250</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>331</v>
+        <v>271</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>311</v>
+        <v>251</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>358</v>
+        <v>298</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>312</v>
+        <v>252</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.5">
       <c r="A24" s="2" t="s">
-        <v>332</v>
+        <v>272</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>313</v>
+        <v>253</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.5">
       <c r="A25" s="2" t="s">
-        <v>360</v>
+        <v>300</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>314</v>
+        <v>254</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.5">
       <c r="A26" s="2" t="s">
-        <v>361</v>
+        <v>301</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>315</v>
+        <v>255</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.5">
       <c r="A27" s="2" t="s">
-        <v>362</v>
+        <v>302</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>316</v>
+        <v>256</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.5">
       <c r="A28" s="2" t="s">
-        <v>363</v>
+        <v>303</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>317</v>
+        <v>257</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.5">
       <c r="A29" s="2" t="s">
-        <v>364</v>
+        <v>304</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>318</v>
+        <v>258</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.5">
       <c r="A30" s="2" t="s">
-        <v>365</v>
+        <v>305</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>319</v>
+        <v>259</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.5">
       <c r="A31" s="2" t="s">
-        <v>366</v>
+        <v>306</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>320</v>
+        <v>260</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.5">
       <c r="A32" s="2" t="s">
-        <v>367</v>
+        <v>307</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>321</v>
+        <v>261</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.5">
       <c r="A33" s="2" t="s">
-        <v>368</v>
+        <v>308</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>322</v>
+        <v>262</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.5">
       <c r="A34" s="2" t="s">
-        <v>369</v>
+        <v>309</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>323</v>
+        <v>263</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.5">
       <c r="A35" s="2" t="s">
-        <v>370</v>
+        <v>310</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>324</v>
+        <v>264</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.5">
       <c r="A36" s="2" t="s">
-        <v>371</v>
+        <v>311</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>325</v>
+        <v>265</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.5">
       <c r="A37" s="2" t="s">
-        <v>372</v>
+        <v>312</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>326</v>
+        <v>266</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.5">
       <c r="A38" s="2" t="s">
-        <v>373</v>
+        <v>313</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>327</v>
+        <v>267</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.5">
       <c r="A39" s="2" t="s">
-        <v>374</v>
+        <v>314</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>333</v>
+        <v>273</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.5">
       <c r="A40" s="2" t="s">
-        <v>375</v>
+        <v>315</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>334</v>
+        <v>274</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.5">
       <c r="A41" s="2" t="s">
-        <v>376</v>
+        <v>316</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>335</v>
+        <v>275</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.5">
       <c r="A42" s="2" t="s">
-        <v>377</v>
+        <v>317</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>336</v>
+        <v>276</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.5">
       <c r="A43" s="2" t="s">
-        <v>378</v>
+        <v>318</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>337</v>
+        <v>277</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.5">
       <c r="A44" s="2" t="s">
-        <v>351</v>
+        <v>291</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>338</v>
+        <v>278</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.5">
       <c r="A45" s="2" t="s">
-        <v>379</v>
+        <v>319</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>339</v>
+        <v>279</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.5">
       <c r="A46" s="2" t="s">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>340</v>
+        <v>280</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.5">
       <c r="A47" s="2" t="s">
-        <v>381</v>
+        <v>321</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>341</v>
+        <v>281</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.5">
       <c r="A48" s="2" t="s">
-        <v>382</v>
+        <v>322</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>342</v>
+        <v>282</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.5">
       <c r="A49" s="2" t="s">
-        <v>383</v>
+        <v>323</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>343</v>
+        <v>283</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.5">
       <c r="A50" s="2" t="s">
-        <v>352</v>
+        <v>292</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>3</v>
@@ -2368,135 +2187,135 @@
     </row>
     <row r="51" spans="1:2" ht="14.5">
       <c r="A51" s="2" t="s">
-        <v>353</v>
+        <v>293</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>344</v>
+        <v>284</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.5">
       <c r="A52" s="2" t="s">
-        <v>354</v>
+        <v>294</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>345</v>
+        <v>285</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.5">
       <c r="A53" s="2" t="s">
-        <v>355</v>
+        <v>295</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>407</v>
+        <v>347</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.5">
       <c r="A54" s="2" t="s">
-        <v>356</v>
+        <v>296</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>346</v>
+        <v>286</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.5">
       <c r="A55" s="2" t="s">
-        <v>384</v>
+        <v>324</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>347</v>
+        <v>287</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="14.5">
       <c r="A56" s="2" t="s">
-        <v>357</v>
+        <v>297</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>348</v>
+        <v>288</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.5">
       <c r="A57" s="2" t="s">
-        <v>385</v>
+        <v>325</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>349</v>
+        <v>289</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="14.5">
       <c r="A58" s="2" t="s">
-        <v>389</v>
+        <v>329</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>390</v>
+        <v>330</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.5">
       <c r="A59" s="2" t="s">
-        <v>391</v>
+        <v>331</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>392</v>
+        <v>332</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="14.5">
       <c r="A60" s="2" t="s">
-        <v>393</v>
+        <v>333</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>394</v>
+        <v>334</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="14.5">
       <c r="A61" s="2" t="s">
-        <v>395</v>
+        <v>335</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>396</v>
+        <v>336</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="14.5">
       <c r="A62" s="2" t="s">
-        <v>397</v>
+        <v>337</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>398</v>
+        <v>338</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="14.5">
       <c r="A63" s="2" t="s">
-        <v>399</v>
+        <v>339</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>400</v>
+        <v>340</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="14.5">
       <c r="A64" s="2" t="s">
-        <v>401</v>
+        <v>341</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>402</v>
+        <v>342</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="14.5">
       <c r="A65" s="2" t="s">
-        <v>403</v>
+        <v>343</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>404</v>
+        <v>344</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="14.5">
       <c r="A66" s="2" t="s">
-        <v>405</v>
+        <v>345</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>406</v>
+        <v>346</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="14.5">
       <c r="A67" s="2" t="s">
-        <v>352</v>
+        <v>292</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>3</v>
@@ -2504,290 +2323,290 @@
     </row>
     <row r="68" spans="1:2" ht="14.5">
       <c r="A68" s="2" t="s">
-        <v>353</v>
+        <v>293</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>344</v>
+        <v>284</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="14.5">
       <c r="A69" s="2" t="s">
-        <v>354</v>
+        <v>294</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>345</v>
+        <v>285</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="14.5">
       <c r="A70" s="2" t="s">
-        <v>355</v>
+        <v>295</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>407</v>
+        <v>347</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="14.5">
       <c r="A71" s="2" t="s">
-        <v>356</v>
+        <v>296</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>346</v>
+        <v>286</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="14.5">
       <c r="A72" s="2" t="s">
-        <v>382</v>
+        <v>322</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>408</v>
+        <v>348</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="14.5">
       <c r="A73" s="2" t="s">
-        <v>383</v>
+        <v>323</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>343</v>
+        <v>283</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="14.5">
       <c r="A74" s="2" t="s">
-        <v>425</v>
+        <v>365</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>409</v>
+        <v>349</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="14.5">
       <c r="A75" s="2" t="s">
-        <v>426</v>
+        <v>366</v>
       </c>
       <c r="B75" s="15" t="s">
-        <v>410</v>
+        <v>350</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="14.5">
       <c r="A76" s="2" t="s">
-        <v>427</v>
+        <v>367</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>411</v>
+        <v>351</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="14.5">
       <c r="A77" s="2" t="s">
-        <v>428</v>
+        <v>368</v>
       </c>
       <c r="B77" s="15" t="s">
-        <v>412</v>
+        <v>352</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="14.5">
       <c r="A78" s="2" t="s">
-        <v>429</v>
+        <v>369</v>
       </c>
       <c r="B78" s="15" t="s">
-        <v>413</v>
+        <v>353</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="14.5">
       <c r="A79" s="2" t="s">
-        <v>430</v>
+        <v>370</v>
       </c>
       <c r="B79" s="15" t="s">
-        <v>414</v>
+        <v>354</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="14.5">
       <c r="A80" s="2" t="s">
-        <v>431</v>
+        <v>371</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>415</v>
+        <v>355</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="14.5">
       <c r="A81" s="2" t="s">
-        <v>432</v>
+        <v>372</v>
       </c>
       <c r="B81" s="15" t="s">
-        <v>416</v>
+        <v>356</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="14.5">
       <c r="A82" s="2" t="s">
-        <v>433</v>
+        <v>373</v>
       </c>
       <c r="B82" s="15" t="s">
-        <v>417</v>
+        <v>357</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="14.5">
       <c r="A83" s="2" t="s">
-        <v>434</v>
+        <v>374</v>
       </c>
       <c r="B83" s="15" t="s">
-        <v>418</v>
+        <v>358</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="14.5">
       <c r="A84" s="2" t="s">
-        <v>435</v>
+        <v>375</v>
       </c>
       <c r="B84" s="15" t="s">
-        <v>419</v>
+        <v>359</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="14.5">
       <c r="A85" s="2" t="s">
-        <v>436</v>
+        <v>376</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>420</v>
+        <v>360</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="14.5">
       <c r="A86" s="2" t="s">
-        <v>439</v>
+        <v>379</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>421</v>
+        <v>361</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="14.5">
       <c r="A87" s="2" t="s">
-        <v>437</v>
+        <v>377</v>
       </c>
       <c r="B87" s="15" t="s">
-        <v>422</v>
+        <v>362</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="14.5">
       <c r="A88" s="2" t="s">
-        <v>438</v>
+        <v>378</v>
       </c>
       <c r="B88" s="15" t="s">
-        <v>423</v>
+        <v>363</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="14.5">
       <c r="A89" s="2" t="s">
-        <v>440</v>
+        <v>380</v>
       </c>
       <c r="B89" s="15" t="s">
-        <v>424</v>
+        <v>364</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="15" customHeight="1">
       <c r="A90" s="2" t="s">
-        <v>479</v>
+        <v>419</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>480</v>
+        <v>420</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="14.5">
       <c r="A91" s="2" t="s">
-        <v>493</v>
+        <v>433</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>481</v>
+        <v>421</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="14.5">
       <c r="A92" s="2" t="s">
-        <v>499</v>
+        <v>439</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>482</v>
+        <v>422</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="14.5">
       <c r="A93" s="2" t="s">
-        <v>498</v>
+        <v>438</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>483</v>
+        <v>423</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="14.5">
       <c r="A94" s="2" t="s">
-        <v>494</v>
+        <v>434</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>484</v>
+        <v>424</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="14.5">
       <c r="A95" s="2" t="s">
-        <v>500</v>
+        <v>440</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>485</v>
+        <v>425</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="14.5">
       <c r="A96" s="2" t="s">
-        <v>501</v>
+        <v>441</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>486</v>
+        <v>426</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="14.5">
       <c r="A97" s="2" t="s">
-        <v>502</v>
+        <v>442</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>487</v>
+        <v>427</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="14.5">
       <c r="A98" s="2" t="s">
-        <v>503</v>
+        <v>443</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>488</v>
+        <v>428</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="14.5">
       <c r="A99" s="2" t="s">
-        <v>504</v>
+        <v>444</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>489</v>
+        <v>429</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="14.5">
       <c r="A100" s="2" t="s">
-        <v>384</v>
+        <v>324</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>347</v>
+        <v>287</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="14.5">
       <c r="A101" s="2" t="s">
-        <v>495</v>
+        <v>435</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>490</v>
+        <v>430</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="14.5">
       <c r="A102" s="2" t="s">
-        <v>496</v>
+        <v>436</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>491</v>
+        <v>431</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="14.5">
       <c r="A103" s="2" t="s">
-        <v>497</v>
+        <v>437</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>492</v>
+        <v>432</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="14.5">
@@ -2796,50 +2615,50 @@
     </row>
     <row r="106" spans="1:2" ht="14.5">
       <c r="A106" t="s">
-        <v>448</v>
+        <v>388</v>
       </c>
       <c r="B106" t="s">
-        <v>449</v>
+        <v>389</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="15" customHeight="1">
       <c r="A107" t="s">
-        <v>451</v>
+        <v>391</v>
       </c>
       <c r="B107" t="s">
-        <v>450</v>
+        <v>390</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="14.5">
       <c r="A108" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="B108" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="14.5">
       <c r="A109" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="B109" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="14.5">
       <c r="A110" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="B110" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="14.5">
       <c r="A111" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="B111" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="14.25" customHeight="1"/>
@@ -2865,7 +2684,7 @@
         <v>49</v>
       </c>
       <c r="B116" t="s">
-        <v>442</v>
+        <v>382</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="14.25" customHeight="1">
@@ -2873,13 +2692,13 @@
         <v>66</v>
       </c>
       <c r="B117" t="s">
-        <v>441</v>
+        <v>381</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="119" spans="1:2" ht="14.25" customHeight="1">
       <c r="A119" t="s">
-        <v>445</v>
+        <v>385</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="15" customHeight="1">
@@ -2916,42 +2735,42 @@
     </row>
     <row r="126" spans="1:2" ht="14.5">
       <c r="A126" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B126" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="14.5">
       <c r="A127" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="B127" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="14.5">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="B128" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="14.5">
       <c r="A129" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="B129" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="14.5">
       <c r="A130" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="B130" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="14.5">
@@ -2988,18 +2807,18 @@
     </row>
     <row r="135" spans="1:2" s="13" customFormat="1" ht="14.5">
       <c r="A135" s="13" t="s">
-        <v>280</v>
+        <v>220</v>
       </c>
       <c r="B135" s="13" t="s">
-        <v>282</v>
+        <v>222</v>
       </c>
     </row>
     <row r="136" spans="1:2" s="13" customFormat="1" ht="14.5">
       <c r="A136" s="13" t="s">
-        <v>281</v>
+        <v>221</v>
       </c>
       <c r="B136" s="13" t="s">
-        <v>283</v>
+        <v>223</v>
       </c>
     </row>
     <row r="137" spans="1:2" s="13" customFormat="1" ht="14.25" customHeight="1">
@@ -3015,31 +2834,31 @@
         <v>124</v>
       </c>
       <c r="B138" s="13" t="s">
-        <v>238</v>
+        <v>193</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="14.25" customHeight="1">
       <c r="A139" t="s">
-        <v>284</v>
+        <v>224</v>
       </c>
       <c r="B139" t="s">
-        <v>225</v>
+        <v>180</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="14.25" customHeight="1">
       <c r="A140" t="s">
-        <v>223</v>
+        <v>178</v>
       </c>
       <c r="B140" t="s">
-        <v>224</v>
+        <v>179</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="14.5">
       <c r="A141" s="2" t="s">
-        <v>226</v>
+        <v>181</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>228</v>
+        <v>183</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="14.5">
@@ -3047,127 +2866,127 @@
         <v>128</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>227</v>
+        <v>182</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="14.5">
       <c r="A143" s="2" t="s">
-        <v>229</v>
+        <v>184</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>266</v>
+        <v>209</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="14.5">
       <c r="A144" s="2" t="s">
-        <v>230</v>
+        <v>185</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>232</v>
+        <v>187</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="14.5">
       <c r="A145" s="2" t="s">
-        <v>231</v>
+        <v>186</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>239</v>
+        <v>194</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="14.5">
       <c r="A146" s="2" t="s">
-        <v>234</v>
+        <v>189</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>233</v>
+        <v>188</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="14.5">
       <c r="A147" s="2" t="s">
-        <v>235</v>
+        <v>190</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>240</v>
+        <v>195</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="14.5">
       <c r="A148" s="2" t="s">
-        <v>236</v>
+        <v>191</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>237</v>
+        <v>192</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="14.5">
       <c r="A149" s="2" t="s">
-        <v>252</v>
+        <v>207</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>245</v>
+        <v>200</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="14.5">
       <c r="A150" s="2" t="s">
-        <v>241</v>
+        <v>196</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>242</v>
+        <v>197</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="14.5">
       <c r="A151" s="2" t="s">
-        <v>243</v>
+        <v>198</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>244</v>
+        <v>199</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="14.5">
       <c r="A152" s="2" t="s">
-        <v>247</v>
+        <v>202</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>246</v>
+        <v>201</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="14.5">
       <c r="A153" s="2" t="s">
-        <v>248</v>
+        <v>203</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>249</v>
+        <v>204</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="14.5">
       <c r="A154" s="2" t="s">
-        <v>250</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>267</v>
+        <v>210</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="14.5">
       <c r="A155" s="2" t="s">
-        <v>251</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>268</v>
+        <v>211</v>
       </c>
     </row>
     <row r="156" spans="1:2" s="13" customFormat="1" ht="14.5">
       <c r="A156" s="14" t="s">
-        <v>287</v>
+        <v>227</v>
       </c>
       <c r="B156" s="14" t="s">
-        <v>289</v>
+        <v>229</v>
       </c>
     </row>
     <row r="157" spans="1:2" s="13" customFormat="1" ht="14.5">
       <c r="A157" s="14" t="s">
-        <v>288</v>
+        <v>228</v>
       </c>
       <c r="B157" s="14" t="s">
-        <v>290</v>
+        <v>230</v>
       </c>
     </row>
     <row r="158" spans="1:2" ht="14.5">
@@ -3216,7 +3035,7 @@
     </row>
     <row r="164" spans="1:3" s="13" customFormat="1" ht="14.25" customHeight="1">
       <c r="A164" s="14" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="B164" s="14" t="s">
         <v>113</v>
@@ -3224,18 +3043,18 @@
     </row>
     <row r="165" spans="1:3" s="13" customFormat="1" ht="14.25" customHeight="1">
       <c r="A165" s="13" t="s">
-        <v>285</v>
+        <v>225</v>
       </c>
       <c r="B165" s="13" t="s">
-        <v>286</v>
+        <v>226</v>
       </c>
     </row>
     <row r="166" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
       <c r="A166" s="9" t="s">
-        <v>192</v>
+        <v>173</v>
       </c>
       <c r="B166" s="9" t="s">
-        <v>193</v>
+        <v>174</v>
       </c>
     </row>
     <row r="167" spans="1:3" ht="14.25" customHeight="1">
@@ -3493,7 +3312,7 @@
         <v>121</v>
       </c>
       <c r="B201" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
     </row>
     <row r="202" spans="1:3" ht="14.25" customHeight="1">
@@ -3548,7 +3367,7 @@
     </row>
     <row r="208" spans="1:3" ht="14.25" customHeight="1">
       <c r="A208" t="s">
-        <v>270</v>
+        <v>213</v>
       </c>
       <c r="B208">
         <v>5</v>
@@ -3559,7 +3378,7 @@
     </row>
     <row r="209" spans="1:3" ht="14.25" customHeight="1">
       <c r="A209" t="s">
-        <v>271</v>
+        <v>214</v>
       </c>
       <c r="B209">
         <v>5</v>
@@ -3570,7 +3389,7 @@
     </row>
     <row r="210" spans="1:3" ht="14.5" customHeight="1">
       <c r="A210" t="s">
-        <v>261</v>
+        <v>208</v>
       </c>
       <c r="B210">
         <v>5</v>
@@ -3689,7 +3508,7 @@
         <v>136</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>279</v>
+        <v>219</v>
       </c>
       <c r="C227" s="6" t="s">
         <v>45</v>
@@ -3700,7 +3519,7 @@
         <v>137</v>
       </c>
       <c r="B228" s="7" t="s">
-        <v>446</v>
+        <v>386</v>
       </c>
       <c r="C228" s="6"/>
     </row>
@@ -3709,7 +3528,7 @@
         <v>138</v>
       </c>
       <c r="B229" s="8" t="s">
-        <v>447</v>
+        <v>387</v>
       </c>
       <c r="C229" s="6"/>
     </row>
@@ -3739,7 +3558,7 @@
         <v>139</v>
       </c>
       <c r="B233" s="5" t="s">
-        <v>279</v>
+        <v>219</v>
       </c>
       <c r="C233" s="6" t="s">
         <v>45</v>
@@ -3750,7 +3569,7 @@
         <v>140</v>
       </c>
       <c r="B234" s="7" t="s">
-        <v>209</v>
+        <v>175</v>
       </c>
     </row>
     <row r="235" spans="1:3" ht="14.25" customHeight="1">
@@ -3766,26 +3585,26 @@
     <row r="238" spans="1:3" ht="14" customHeight="1"/>
     <row r="239" spans="1:3" ht="14" customHeight="1">
       <c r="A239" t="s">
-        <v>212</v>
+        <v>176</v>
       </c>
       <c r="B239" t="s">
-        <v>213</v>
+        <v>177</v>
       </c>
     </row>
     <row r="240" spans="1:3" ht="14" customHeight="1">
       <c r="A240" t="s">
-        <v>272</v>
+        <v>215</v>
       </c>
       <c r="B240" t="s">
-        <v>273</v>
+        <v>216</v>
       </c>
     </row>
     <row r="241" spans="1:3" ht="14" customHeight="1">
       <c r="A241" t="s">
-        <v>274</v>
+        <v>217</v>
       </c>
       <c r="B241" t="s">
-        <v>275</v>
+        <v>218</v>
       </c>
     </row>
     <row r="242" spans="1:3" ht="14" customHeight="1"/>
@@ -3815,7 +3634,7 @@
     </row>
     <row r="256" spans="1:3" ht="14.25" customHeight="1">
       <c r="A256" t="s">
-        <v>291</v>
+        <v>231</v>
       </c>
       <c r="B256" s="2">
         <v>5</v>
@@ -3826,7 +3645,7 @@
     </row>
     <row r="257" spans="1:3" ht="14.25" customHeight="1">
       <c r="A257" t="s">
-        <v>292</v>
+        <v>232</v>
       </c>
       <c r="B257" s="2">
         <v>5</v>
@@ -3837,7 +3656,7 @@
     </row>
     <row r="258" spans="1:3" ht="14.25" customHeight="1">
       <c r="A258" t="s">
-        <v>295</v>
+        <v>235</v>
       </c>
       <c r="B258" s="2">
         <v>5</v>
@@ -3856,34 +3675,34 @@
     <row r="267" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="268" spans="1:3" ht="14.25" customHeight="1">
       <c r="A268" t="s">
-        <v>293</v>
+        <v>233</v>
       </c>
       <c r="B268" t="s">
-        <v>297</v>
+        <v>237</v>
       </c>
     </row>
     <row r="269" spans="1:3" ht="14.25" customHeight="1">
       <c r="A269" t="s">
-        <v>294</v>
+        <v>234</v>
       </c>
       <c r="B269" t="s">
-        <v>298</v>
+        <v>238</v>
       </c>
     </row>
     <row r="270" spans="1:3" ht="14.25" customHeight="1">
       <c r="A270" t="s">
-        <v>296</v>
+        <v>236</v>
       </c>
       <c r="B270" t="s">
-        <v>299</v>
+        <v>239</v>
       </c>
     </row>
     <row r="271" spans="1:3" ht="14.25" customHeight="1">
       <c r="A271" t="s">
-        <v>387</v>
+        <v>327</v>
       </c>
       <c r="B271" t="s">
-        <v>388</v>
+        <v>328</v>
       </c>
     </row>
     <row r="272" spans="1:3" ht="14.25" customHeight="1"/>
@@ -3891,7 +3710,7 @@
     <row r="274" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="275" spans="1:3" ht="14.25" customHeight="1">
       <c r="A275" t="s">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="B275">
         <v>5</v>
@@ -3902,17 +3721,17 @@
     </row>
     <row r="276" spans="1:3" ht="14.25" customHeight="1">
       <c r="A276" t="s">
-        <v>301</v>
+        <v>241</v>
       </c>
       <c r="B276" t="s">
-        <v>302</v>
+        <v>242</v>
       </c>
     </row>
     <row r="277" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="278" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="279" spans="1:3" ht="14.25" customHeight="1">
       <c r="A279" t="s">
-        <v>303</v>
+        <v>243</v>
       </c>
       <c r="B279">
         <v>5</v>
@@ -3925,7 +3744,7 @@
     <row r="281" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="282" spans="1:3" ht="14" customHeight="1">
       <c r="A282" t="s">
-        <v>455</v>
+        <v>395</v>
       </c>
       <c r="B282">
         <v>100</v>
@@ -3936,7 +3755,7 @@
     </row>
     <row r="283" spans="1:3" ht="14.25" customHeight="1">
       <c r="A283" t="s">
-        <v>454</v>
+        <v>394</v>
       </c>
       <c r="B283">
         <v>100</v>
@@ -3947,7 +3766,7 @@
     </row>
     <row r="284" spans="1:3" ht="14.25" customHeight="1">
       <c r="A284" t="s">
-        <v>458</v>
+        <v>398</v>
       </c>
       <c r="B284">
         <v>100</v>
@@ -3958,7 +3777,7 @@
     </row>
     <row r="285" spans="1:3" ht="14.25" customHeight="1">
       <c r="A285" t="s">
-        <v>461</v>
+        <v>401</v>
       </c>
       <c r="B285">
         <v>100</v>
@@ -3969,7 +3788,7 @@
     </row>
     <row r="286" spans="1:3" ht="14.25" customHeight="1">
       <c r="A286" t="s">
-        <v>464</v>
+        <v>404</v>
       </c>
       <c r="B286">
         <v>100</v>
@@ -3980,7 +3799,7 @@
     </row>
     <row r="287" spans="1:3" ht="14.25" customHeight="1">
       <c r="A287" t="s">
-        <v>467</v>
+        <v>407</v>
       </c>
       <c r="B287">
         <v>100</v>
@@ -3991,7 +3810,7 @@
     </row>
     <row r="288" spans="1:3" ht="14.25" customHeight="1">
       <c r="A288" t="s">
-        <v>470</v>
+        <v>410</v>
       </c>
       <c r="B288">
         <v>100</v>
@@ -4002,7 +3821,7 @@
     </row>
     <row r="289" spans="1:3" ht="14.25" customHeight="1">
       <c r="A289" t="s">
-        <v>473</v>
+        <v>413</v>
       </c>
       <c r="B289">
         <v>100</v>
@@ -4013,7 +3832,7 @@
     </row>
     <row r="290" spans="1:3" ht="14.25" customHeight="1">
       <c r="A290" t="s">
-        <v>476</v>
+        <v>416</v>
       </c>
       <c r="B290">
         <v>100</v>
@@ -4028,74 +3847,74 @@
     <row r="294" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="295" spans="1:3" ht="14.25" customHeight="1">
       <c r="A295" t="s">
-        <v>452</v>
+        <v>392</v>
       </c>
       <c r="B295" t="s">
-        <v>453</v>
+        <v>393</v>
       </c>
     </row>
     <row r="296" spans="1:3" ht="14.25" customHeight="1">
       <c r="A296" t="s">
-        <v>456</v>
+        <v>396</v>
       </c>
       <c r="B296" t="s">
-        <v>457</v>
+        <v>397</v>
       </c>
     </row>
     <row r="297" spans="1:3" ht="14.25" customHeight="1">
       <c r="A297" t="s">
-        <v>459</v>
+        <v>399</v>
       </c>
       <c r="B297" t="s">
-        <v>460</v>
+        <v>400</v>
       </c>
     </row>
     <row r="298" spans="1:3" ht="14.25" customHeight="1">
       <c r="A298" t="s">
-        <v>462</v>
+        <v>402</v>
       </c>
       <c r="B298" t="s">
-        <v>463</v>
+        <v>403</v>
       </c>
     </row>
     <row r="299" spans="1:3" ht="14.25" customHeight="1">
       <c r="A299" t="s">
-        <v>465</v>
+        <v>405</v>
       </c>
       <c r="B299" t="s">
-        <v>466</v>
+        <v>406</v>
       </c>
     </row>
     <row r="300" spans="1:3" ht="14.25" customHeight="1">
       <c r="A300" t="s">
-        <v>468</v>
+        <v>408</v>
       </c>
       <c r="B300" t="s">
-        <v>469</v>
+        <v>409</v>
       </c>
     </row>
     <row r="301" spans="1:3" ht="14.25" customHeight="1">
       <c r="A301" t="s">
-        <v>471</v>
+        <v>411</v>
       </c>
       <c r="B301" t="s">
-        <v>472</v>
+        <v>412</v>
       </c>
     </row>
     <row r="302" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="A302" s="6" t="s">
-        <v>474</v>
+        <v>414</v>
       </c>
       <c r="B302" s="6" t="s">
-        <v>475</v>
+        <v>415</v>
       </c>
     </row>
     <row r="303" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="A303" s="6" t="s">
-        <v>477</v>
+        <v>417</v>
       </c>
       <c r="B303" s="7" t="s">
-        <v>478</v>
+        <v>418</v>
       </c>
     </row>
     <row r="304" spans="1:3" s="6" customFormat="1" ht="14.5">
@@ -5224,7 +5043,7 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>269</v>
+        <v>212</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
@@ -7256,2276 +7075,4 @@
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2E1777-460A-49FA-8ECC-5B7815DCE559}">
-  <dimension ref="A1:Z1079"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="49.54296875" customWidth="1"/>
-    <col min="2" max="2" width="72.7265625" customWidth="1"/>
-    <col min="3" max="3" width="22.6328125" customWidth="1"/>
-    <col min="4" max="26" width="8.6328125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-    </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:26" ht="15" customHeight="1">
-      <c r="A3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B4">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" ht="14.5">
-      <c r="A5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5">
-        <v>1000</v>
-      </c>
-      <c r="C5" s="4"/>
-    </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B8" s="9">
-        <v>0</v>
-      </c>
-      <c r="C8" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" t="s">
-        <v>153</v>
-      </c>
-      <c r="B12" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" ht="15" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:26" ht="15" customHeight="1">
-      <c r="A15" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" ht="15" customHeight="1">
-      <c r="A16" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15" customHeight="1">
-      <c r="A20" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15" customHeight="1">
-      <c r="A21" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15" customHeight="1">
-      <c r="A22" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="14.5">
-      <c r="A23" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="14.5">
-      <c r="A24" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="14.5">
-      <c r="A26" t="s">
-        <v>205</v>
-      </c>
-      <c r="B26" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="15" customHeight="1">
-      <c r="A27" t="s">
-        <v>163</v>
-      </c>
-      <c r="B27" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="14.5">
-      <c r="A28" t="s">
-        <v>164</v>
-      </c>
-      <c r="B28" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="14.5">
-      <c r="A29" t="s">
-        <v>172</v>
-      </c>
-      <c r="B29" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="14.5">
-      <c r="A30" t="s">
-        <v>173</v>
-      </c>
-      <c r="B30" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="14.5">
-      <c r="A31" t="s">
-        <v>174</v>
-      </c>
-      <c r="B31" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="33" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A33" t="s">
-        <v>129</v>
-      </c>
-      <c r="B33" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A34" t="s">
-        <v>67</v>
-      </c>
-      <c r="B34" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="36" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A36" t="s">
-        <v>49</v>
-      </c>
-      <c r="B36" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A37" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="15" customHeight="1">
-      <c r="A39" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="15" customHeight="1">
-      <c r="A40" t="s">
-        <v>64</v>
-      </c>
-      <c r="B40" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="15" customHeight="1">
-      <c r="A41" t="s">
-        <v>65</v>
-      </c>
-      <c r="B41" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A43" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="B43" s="11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="14.5">
-      <c r="A44" t="s">
-        <v>156</v>
-      </c>
-      <c r="B44" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="14.5">
-      <c r="A45" t="s">
-        <v>180</v>
-      </c>
-      <c r="B45" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="14.5">
-      <c r="A46" t="s">
-        <v>178</v>
-      </c>
-      <c r="B46" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="14.5">
-      <c r="A47" t="s">
-        <v>182</v>
-      </c>
-      <c r="B47" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="14.5">
-      <c r="A48" t="s">
-        <v>184</v>
-      </c>
-      <c r="B48" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="14.5">
-      <c r="A49" t="s">
-        <v>145</v>
-      </c>
-      <c r="B49" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="14.5">
-      <c r="A50" t="s">
-        <v>147</v>
-      </c>
-      <c r="B50" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="14.5">
-      <c r="A51" t="s">
-        <v>94</v>
-      </c>
-      <c r="B51" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="14.5">
-      <c r="A52" t="s">
-        <v>149</v>
-      </c>
-      <c r="B52" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="14.5">
-      <c r="A53" t="s">
-        <v>188</v>
-      </c>
-      <c r="B53" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="14.5">
-      <c r="A54" t="s">
-        <v>190</v>
-      </c>
-      <c r="B54" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A55" t="s">
-        <v>123</v>
-      </c>
-      <c r="B55" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A56" t="s">
-        <v>124</v>
-      </c>
-      <c r="B56" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A57" t="s">
-        <v>220</v>
-      </c>
-      <c r="B57" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A58" t="s">
-        <v>223</v>
-      </c>
-      <c r="B58" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="14.5">
-      <c r="A59" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="14.5">
-      <c r="A60" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" ht="14.5">
-      <c r="A61" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" ht="14.5">
-      <c r="A62" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" ht="14.5">
-      <c r="A63" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="14.5">
-      <c r="A64" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="14.5">
-      <c r="A65" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" ht="14.5">
-      <c r="A66" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" ht="14.5">
-      <c r="A67" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="14.5">
-      <c r="A68" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" ht="14.5">
-      <c r="A69" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" ht="14.5">
-      <c r="A70" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" ht="14.5">
-      <c r="A71" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" ht="14.5">
-      <c r="A72" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" ht="14.5">
-      <c r="A73" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" ht="14.5">
-      <c r="A74" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" ht="14.5">
-      <c r="A75" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" ht="14.5">
-      <c r="A76" s="2"/>
-      <c r="B76" s="2"/>
-    </row>
-    <row r="77" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A77" t="s">
-        <v>88</v>
-      </c>
-      <c r="B77" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A78" t="s">
-        <v>95</v>
-      </c>
-      <c r="B78" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A79" t="s">
-        <v>89</v>
-      </c>
-      <c r="B79" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A80" t="s">
-        <v>104</v>
-      </c>
-      <c r="B80" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A81" t="s">
-        <v>108</v>
-      </c>
-      <c r="B81" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A82" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A83" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="B83" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A84" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="B84" s="9" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A85" s="2"/>
-      <c r="B85" s="2"/>
-    </row>
-    <row r="86" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A86" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B86" s="7">
-        <v>2000</v>
-      </c>
-      <c r="C86" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A87" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B87">
-        <v>1</v>
-      </c>
-      <c r="C87" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A88" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B88" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="C88" s="6"/>
-    </row>
-    <row r="89" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A89" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B89" s="7">
-        <v>3</v>
-      </c>
-      <c r="C89" s="6"/>
-    </row>
-    <row r="90" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A90" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B90" s="7">
-        <v>3</v>
-      </c>
-      <c r="C90" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" ht="14.5"/>
-    <row r="92" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A92" t="s">
-        <v>91</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="94" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A94" t="s">
-        <v>109</v>
-      </c>
-      <c r="B94" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A95" t="s">
-        <v>97</v>
-      </c>
-      <c r="B95" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="97" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A97" t="s">
-        <v>111</v>
-      </c>
-      <c r="B97" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A98" t="s">
-        <v>117</v>
-      </c>
-      <c r="B98" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A99" t="s">
-        <v>112</v>
-      </c>
-      <c r="B99" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A100" t="s">
-        <v>118</v>
-      </c>
-      <c r="B100" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="102" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A102" t="s">
-        <v>115</v>
-      </c>
-      <c r="B102">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A103" t="s">
-        <v>116</v>
-      </c>
-      <c r="B103">
-        <v>40000</v>
-      </c>
-      <c r="C103" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A104" s="6"/>
-      <c r="B104" s="7"/>
-    </row>
-    <row r="105" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A105" t="s">
-        <v>106</v>
-      </c>
-      <c r="B105">
-        <v>30000</v>
-      </c>
-      <c r="C105" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A106" t="s">
-        <v>103</v>
-      </c>
-      <c r="B106">
-        <v>30000</v>
-      </c>
-      <c r="C106" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A107" t="s">
-        <v>107</v>
-      </c>
-      <c r="B107">
-        <v>60000</v>
-      </c>
-      <c r="C107" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A108" s="6"/>
-      <c r="B108" s="7"/>
-      <c r="C108" s="6"/>
-    </row>
-    <row r="109" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A109" t="s">
-        <v>74</v>
-      </c>
-      <c r="B109">
-        <v>2000</v>
-      </c>
-      <c r="C109" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A110" t="s">
-        <v>76</v>
-      </c>
-      <c r="B110">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A111" t="s">
-        <v>77</v>
-      </c>
-      <c r="B111">
-        <v>1</v>
-      </c>
-      <c r="C111" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="113" spans="1:3" ht="15" customHeight="1">
-      <c r="A113" t="s">
-        <v>75</v>
-      </c>
-      <c r="B113">
-        <v>2000</v>
-      </c>
-      <c r="C113" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A114" t="s">
-        <v>78</v>
-      </c>
-      <c r="B114">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" ht="17.5" customHeight="1">
-      <c r="A115" t="s">
-        <v>79</v>
-      </c>
-      <c r="B115">
-        <v>1</v>
-      </c>
-      <c r="C115" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="117" spans="1:3" ht="17.5" customHeight="1">
-      <c r="A117" t="s">
-        <v>151</v>
-      </c>
-      <c r="B117">
-        <v>3000</v>
-      </c>
-      <c r="C117" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="119" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A119" t="s">
-        <v>121</v>
-      </c>
-      <c r="B119" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A120" s="6"/>
-      <c r="B120" s="7"/>
-      <c r="C120" s="6"/>
-    </row>
-    <row r="121" spans="1:3" ht="14" customHeight="1">
-      <c r="A121" t="s">
-        <v>122</v>
-      </c>
-      <c r="B121">
-        <v>1</v>
-      </c>
-      <c r="C121" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="123" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A123" t="s">
-        <v>134</v>
-      </c>
-      <c r="B123">
-        <v>60000</v>
-      </c>
-      <c r="C123" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A124" t="s">
-        <v>133</v>
-      </c>
-      <c r="B124">
-        <v>60000</v>
-      </c>
-      <c r="C124" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A125" t="s">
-        <v>135</v>
-      </c>
-      <c r="B125">
-        <v>60000</v>
-      </c>
-      <c r="C125" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A126" t="s">
-        <v>270</v>
-      </c>
-      <c r="B126">
-        <v>5</v>
-      </c>
-      <c r="C126" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A127" t="s">
-        <v>271</v>
-      </c>
-      <c r="B127">
-        <v>5</v>
-      </c>
-      <c r="C127" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" ht="14.5" customHeight="1">
-      <c r="A128" t="s">
-        <v>261</v>
-      </c>
-      <c r="B128">
-        <v>5</v>
-      </c>
-      <c r="C128" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="130" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A130" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B130" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="132" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A132" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B132" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A133" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B133" s="7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A134" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B134" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A135" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B135" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="137" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A137" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B137" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A138" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B138" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A139" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B139" s="7">
-        <v>60</v>
-      </c>
-      <c r="C139" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="141" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A141" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B141" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C141" s="6"/>
-    </row>
-    <row r="142" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A142" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B142" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C142" s="6"/>
-    </row>
-    <row r="143" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A143" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B143" s="7">
-        <v>60</v>
-      </c>
-      <c r="C143" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A144" s="6"/>
-      <c r="B144" s="6"/>
-      <c r="C144" s="6"/>
-    </row>
-    <row r="145" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A145" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="B145" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="C145" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A146" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B146" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="C146" s="6"/>
-    </row>
-    <row r="147" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A147" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B147" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="C147" s="6"/>
-    </row>
-    <row r="148" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A148" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B148" s="6"/>
-      <c r="C148" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A149" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B149" s="7">
-        <v>60000</v>
-      </c>
-      <c r="C149" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="151" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A151" t="s">
-        <v>139</v>
-      </c>
-      <c r="B151" s="5" t="s">
-        <v>279</v>
-      </c>
-      <c r="C151" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A152" t="s">
-        <v>140</v>
-      </c>
-      <c r="B152" s="7" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A153" t="s">
-        <v>141</v>
-      </c>
-      <c r="B153" s="8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3" ht="14" customHeight="1"/>
-    <row r="155" spans="1:3" ht="14" customHeight="1">
-      <c r="A155" t="s">
-        <v>210</v>
-      </c>
-      <c r="B155">
-        <v>5</v>
-      </c>
-      <c r="C155" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" ht="14" customHeight="1"/>
-    <row r="157" spans="1:3" ht="14" customHeight="1">
-      <c r="A157" t="s">
-        <v>212</v>
-      </c>
-      <c r="B157" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" ht="14" customHeight="1">
-      <c r="A158" t="s">
-        <v>272</v>
-      </c>
-      <c r="B158" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3" ht="14" customHeight="1">
-      <c r="A159" t="s">
-        <v>274</v>
-      </c>
-      <c r="B159" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3" ht="14" customHeight="1"/>
-    <row r="161" spans="1:3" ht="14" customHeight="1">
-      <c r="A161" t="s">
-        <v>216</v>
-      </c>
-      <c r="B161" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3" ht="14" customHeight="1">
-      <c r="A162" t="s">
-        <v>217</v>
-      </c>
-      <c r="B162" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" ht="14" customHeight="1"/>
-    <row r="164" spans="1:3" ht="15" customHeight="1">
-      <c r="A164" t="s">
-        <v>218</v>
-      </c>
-      <c r="B164" s="12" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A165" t="s">
-        <v>222</v>
-      </c>
-      <c r="B165" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A166" t="s">
-        <v>257</v>
-      </c>
-      <c r="B166" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A167" t="s">
-        <v>258</v>
-      </c>
-      <c r="B167" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="169" spans="1:3" ht="15" customHeight="1">
-      <c r="A169" t="s">
-        <v>262</v>
-      </c>
-      <c r="B169" s="12" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" ht="15" customHeight="1">
-      <c r="A170" t="s">
-        <v>263</v>
-      </c>
-      <c r="B170" s="12" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" ht="15" customHeight="1">
-      <c r="B171" s="12"/>
-    </row>
-    <row r="172" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A172" t="s">
-        <v>276</v>
-      </c>
-      <c r="B172" s="2">
-        <v>25</v>
-      </c>
-      <c r="C172" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3" ht="15" customHeight="1">
-      <c r="B173" s="2"/>
-    </row>
-    <row r="174" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B174" s="2"/>
-    </row>
-    <row r="175" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B175" s="2"/>
-    </row>
-    <row r="176" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="177" ht="14.25" customHeight="1"/>
-    <row r="178" ht="14.25" customHeight="1"/>
-    <row r="179" ht="14.25" customHeight="1"/>
-    <row r="180" ht="14.25" customHeight="1"/>
-    <row r="181" ht="14.25" customHeight="1"/>
-    <row r="182" ht="14.25" customHeight="1"/>
-    <row r="183" ht="14.25" customHeight="1"/>
-    <row r="184" ht="14.25" customHeight="1"/>
-    <row r="185" ht="14.25" customHeight="1"/>
-    <row r="186" ht="14.25" customHeight="1"/>
-    <row r="187" ht="14.25" customHeight="1"/>
-    <row r="188" ht="14.25" customHeight="1"/>
-    <row r="189" ht="14.25" customHeight="1"/>
-    <row r="190" ht="14.25" customHeight="1"/>
-    <row r="191" ht="14.25" customHeight="1"/>
-    <row r="192" ht="14.25" customHeight="1"/>
-    <row r="193" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="194" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="195" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="196" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="197" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="198" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="199" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="200" spans="2:2" s="6" customFormat="1" ht="14.5"/>
-    <row r="201" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B201" s="7"/>
-    </row>
-    <row r="202" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B202" s="7"/>
-    </row>
-    <row r="203" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B203" s="7"/>
-    </row>
-    <row r="204" spans="2:2" s="6" customFormat="1" ht="14.5"/>
-    <row r="205" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B205" s="7"/>
-    </row>
-    <row r="206" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B206" s="7"/>
-    </row>
-    <row r="207" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B207" s="7"/>
-    </row>
-    <row r="208" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="209" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A209" s="6"/>
-      <c r="B209" s="7"/>
-      <c r="C209" s="6"/>
-    </row>
-    <row r="210" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A210" s="6"/>
-      <c r="B210" s="8"/>
-      <c r="C210" s="6"/>
-    </row>
-    <row r="211" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A211" s="6"/>
-      <c r="B211" s="7"/>
-      <c r="C211" s="6"/>
-    </row>
-    <row r="212" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A212" s="6"/>
-      <c r="B212" s="6"/>
-      <c r="C212" s="6"/>
-    </row>
-    <row r="213" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A213" s="6"/>
-      <c r="B213" s="5"/>
-      <c r="C213" s="6"/>
-    </row>
-    <row r="214" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A214" s="6"/>
-      <c r="B214" s="7"/>
-      <c r="C214" s="6"/>
-    </row>
-    <row r="215" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A215" s="6"/>
-      <c r="B215" s="8"/>
-      <c r="C215" s="6"/>
-    </row>
-    <row r="216" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A216" s="6"/>
-      <c r="B216" s="6"/>
-      <c r="C216" s="6"/>
-    </row>
-    <row r="217" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A217" s="6"/>
-      <c r="B217" s="7"/>
-      <c r="C217" s="6"/>
-    </row>
-    <row r="218" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="219" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B219" s="5"/>
-    </row>
-    <row r="220" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B220" s="7"/>
-    </row>
-    <row r="221" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B221" s="8"/>
-    </row>
-    <row r="222" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="223" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A223" s="6"/>
-    </row>
-    <row r="224" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="225" ht="14.25" customHeight="1"/>
-    <row r="226" ht="14.25" customHeight="1"/>
-    <row r="227" ht="14.25" customHeight="1"/>
-    <row r="228" ht="14.25" customHeight="1"/>
-    <row r="229" ht="14.25" customHeight="1"/>
-    <row r="230" ht="14.25" customHeight="1"/>
-    <row r="231" ht="14.25" customHeight="1"/>
-    <row r="232" ht="14.25" customHeight="1"/>
-    <row r="233" ht="14.25" customHeight="1"/>
-    <row r="234" ht="14.25" customHeight="1"/>
-    <row r="235" ht="14.25" customHeight="1"/>
-    <row r="236" ht="14.25" customHeight="1"/>
-    <row r="237" ht="14.25" customHeight="1"/>
-    <row r="238" ht="14.25" customHeight="1"/>
-    <row r="239" ht="14.25" customHeight="1"/>
-    <row r="240" ht="14.25" customHeight="1"/>
-    <row r="241" ht="14.25" customHeight="1"/>
-    <row r="242" ht="14.25" customHeight="1"/>
-    <row r="243" ht="14.25" customHeight="1"/>
-    <row r="244" ht="14.25" customHeight="1"/>
-    <row r="245" ht="14.25" customHeight="1"/>
-    <row r="246" ht="14.25" customHeight="1"/>
-    <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
-    <row r="249" ht="14.25" customHeight="1"/>
-    <row r="250" ht="14.25" customHeight="1"/>
-    <row r="251" ht="14.25" customHeight="1"/>
-    <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1"/>
-    <row r="254" ht="14.25" customHeight="1"/>
-    <row r="255" ht="14.25" customHeight="1"/>
-    <row r="256" ht="14.25" customHeight="1"/>
-    <row r="257" ht="14.25" customHeight="1"/>
-    <row r="258" ht="14.25" customHeight="1"/>
-    <row r="259" ht="14.25" customHeight="1"/>
-    <row r="260" ht="14.25" customHeight="1"/>
-    <row r="261" ht="14.25" customHeight="1"/>
-    <row r="262" ht="14.25" customHeight="1"/>
-    <row r="263" ht="14.25" customHeight="1"/>
-    <row r="264" ht="14.25" customHeight="1"/>
-    <row r="265" ht="14.25" customHeight="1"/>
-    <row r="266" ht="14.25" customHeight="1"/>
-    <row r="267" ht="14.25" customHeight="1"/>
-    <row r="268" ht="14.25" customHeight="1"/>
-    <row r="269" ht="14.25" customHeight="1"/>
-    <row r="270" ht="14.25" customHeight="1"/>
-    <row r="271" ht="14.25" customHeight="1"/>
-    <row r="272" ht="14.25" customHeight="1"/>
-    <row r="273" ht="14.25" customHeight="1"/>
-    <row r="274" ht="14.25" customHeight="1"/>
-    <row r="275" ht="14.25" customHeight="1"/>
-    <row r="276" ht="14.25" customHeight="1"/>
-    <row r="277" ht="14.25" customHeight="1"/>
-    <row r="278" ht="14.25" customHeight="1"/>
-    <row r="279" ht="14.25" customHeight="1"/>
-    <row r="280" ht="14.25" customHeight="1"/>
-    <row r="281" ht="14.25" customHeight="1"/>
-    <row r="282" ht="14.25" customHeight="1"/>
-    <row r="283" ht="14.25" customHeight="1"/>
-    <row r="284" ht="14.25" customHeight="1"/>
-    <row r="285" ht="14.25" customHeight="1"/>
-    <row r="286" ht="14.25" customHeight="1"/>
-    <row r="287" ht="14.25" customHeight="1"/>
-    <row r="288" ht="14.25" customHeight="1"/>
-    <row r="289" ht="14.25" customHeight="1"/>
-    <row r="290" ht="14.25" customHeight="1"/>
-    <row r="291" ht="14.25" customHeight="1"/>
-    <row r="292" ht="14.25" customHeight="1"/>
-    <row r="293" ht="14.25" customHeight="1"/>
-    <row r="294" ht="14.25" customHeight="1"/>
-    <row r="295" ht="14.25" customHeight="1"/>
-    <row r="296" ht="14.25" customHeight="1"/>
-    <row r="297" ht="14.25" customHeight="1"/>
-    <row r="298" ht="14.25" customHeight="1"/>
-    <row r="299" ht="14.25" customHeight="1"/>
-    <row r="300" ht="14.25" customHeight="1"/>
-    <row r="301" ht="14.25" customHeight="1"/>
-    <row r="302" ht="14.25" customHeight="1"/>
-    <row r="303" ht="14.25" customHeight="1"/>
-    <row r="304" ht="14.25" customHeight="1"/>
-    <row r="305" ht="14.25" customHeight="1"/>
-    <row r="306" ht="14.25" customHeight="1"/>
-    <row r="307" ht="14.25" customHeight="1"/>
-    <row r="308" ht="14.25" customHeight="1"/>
-    <row r="309" ht="14.25" customHeight="1"/>
-    <row r="310" ht="14.25" customHeight="1"/>
-    <row r="311" ht="14.25" customHeight="1"/>
-    <row r="312" ht="14.25" customHeight="1"/>
-    <row r="313" ht="14.25" customHeight="1"/>
-    <row r="314" ht="14.25" customHeight="1"/>
-    <row r="315" ht="14.25" customHeight="1"/>
-    <row r="316" ht="14.25" customHeight="1"/>
-    <row r="317" ht="14.25" customHeight="1"/>
-    <row r="318" ht="14.25" customHeight="1"/>
-    <row r="319" ht="14.25" customHeight="1"/>
-    <row r="320" ht="14.25" customHeight="1"/>
-    <row r="321" ht="14.25" customHeight="1"/>
-    <row r="322" ht="14.25" customHeight="1"/>
-    <row r="323" ht="14.25" customHeight="1"/>
-    <row r="324" ht="14.25" customHeight="1"/>
-    <row r="325" ht="14.25" customHeight="1"/>
-    <row r="326" ht="14.25" customHeight="1"/>
-    <row r="327" ht="14.25" customHeight="1"/>
-    <row r="328" ht="14.25" customHeight="1"/>
-    <row r="329" ht="14.25" customHeight="1"/>
-    <row r="330" ht="14.25" customHeight="1"/>
-    <row r="331" ht="14.25" customHeight="1"/>
-    <row r="332" ht="14.25" customHeight="1"/>
-    <row r="333" ht="14.25" customHeight="1"/>
-    <row r="334" ht="14.25" customHeight="1"/>
-    <row r="335" ht="14.25" customHeight="1"/>
-    <row r="336" ht="14.25" customHeight="1"/>
-    <row r="337" ht="14.25" customHeight="1"/>
-    <row r="338" ht="14.25" customHeight="1"/>
-    <row r="339" ht="14.25" customHeight="1"/>
-    <row r="340" ht="14.25" customHeight="1"/>
-    <row r="341" ht="14.25" customHeight="1"/>
-    <row r="342" ht="14.25" customHeight="1"/>
-    <row r="343" ht="14.25" customHeight="1"/>
-    <row r="344" ht="14.25" customHeight="1"/>
-    <row r="345" ht="14.25" customHeight="1"/>
-    <row r="346" ht="14.25" customHeight="1"/>
-    <row r="347" ht="14.25" customHeight="1"/>
-    <row r="348" ht="14.25" customHeight="1"/>
-    <row r="349" ht="14.25" customHeight="1"/>
-    <row r="350" ht="14.25" customHeight="1"/>
-    <row r="351" ht="14.25" customHeight="1"/>
-    <row r="352" ht="14.25" customHeight="1"/>
-    <row r="353" ht="14.25" customHeight="1"/>
-    <row r="354" ht="14.25" customHeight="1"/>
-    <row r="355" ht="14.25" customHeight="1"/>
-    <row r="356" ht="14.25" customHeight="1"/>
-    <row r="357" ht="14.25" customHeight="1"/>
-    <row r="358" ht="14.25" customHeight="1"/>
-    <row r="359" ht="14.25" customHeight="1"/>
-    <row r="360" ht="14.25" customHeight="1"/>
-    <row r="361" ht="14.25" customHeight="1"/>
-    <row r="362" ht="14.25" customHeight="1"/>
-    <row r="363" ht="14.25" customHeight="1"/>
-    <row r="364" ht="14.25" customHeight="1"/>
-    <row r="365" ht="14.25" customHeight="1"/>
-    <row r="366" ht="14.25" customHeight="1"/>
-    <row r="367" ht="14.25" customHeight="1"/>
-    <row r="368" ht="14.25" customHeight="1"/>
-    <row r="369" ht="14.25" customHeight="1"/>
-    <row r="370" ht="14.25" customHeight="1"/>
-    <row r="371" ht="14.25" customHeight="1"/>
-    <row r="372" ht="14.25" customHeight="1"/>
-    <row r="373" ht="14.25" customHeight="1"/>
-    <row r="374" ht="14.25" customHeight="1"/>
-    <row r="375" ht="14.25" customHeight="1"/>
-    <row r="376" ht="14.25" customHeight="1"/>
-    <row r="377" ht="14.25" customHeight="1"/>
-    <row r="378" ht="14.25" customHeight="1"/>
-    <row r="379" ht="14.25" customHeight="1"/>
-    <row r="380" ht="14.25" customHeight="1"/>
-    <row r="381" ht="14.25" customHeight="1"/>
-    <row r="382" ht="14.25" customHeight="1"/>
-    <row r="383" ht="14.25" customHeight="1"/>
-    <row r="384" ht="14.25" customHeight="1"/>
-    <row r="385" ht="14.25" customHeight="1"/>
-    <row r="386" ht="14.25" customHeight="1"/>
-    <row r="387" ht="14.25" customHeight="1"/>
-    <row r="388" ht="14.25" customHeight="1"/>
-    <row r="389" ht="14.25" customHeight="1"/>
-    <row r="390" ht="14.25" customHeight="1"/>
-    <row r="391" ht="14.25" customHeight="1"/>
-    <row r="392" ht="14.25" customHeight="1"/>
-    <row r="393" ht="14.25" customHeight="1"/>
-    <row r="394" ht="14.25" customHeight="1"/>
-    <row r="395" ht="14.25" customHeight="1"/>
-    <row r="396" ht="14.25" customHeight="1"/>
-    <row r="397" ht="14.25" customHeight="1"/>
-    <row r="398" ht="14.25" customHeight="1"/>
-    <row r="399" ht="14.25" customHeight="1"/>
-    <row r="400" ht="14.25" customHeight="1"/>
-    <row r="401" ht="14.25" customHeight="1"/>
-    <row r="402" ht="14.25" customHeight="1"/>
-    <row r="403" ht="14.25" customHeight="1"/>
-    <row r="404" ht="14.25" customHeight="1"/>
-    <row r="405" ht="14.25" customHeight="1"/>
-    <row r="406" ht="14.25" customHeight="1"/>
-    <row r="407" ht="14.25" customHeight="1"/>
-    <row r="408" ht="14.25" customHeight="1"/>
-    <row r="409" ht="14.25" customHeight="1"/>
-    <row r="410" ht="14.25" customHeight="1"/>
-    <row r="411" ht="14.25" customHeight="1"/>
-    <row r="412" ht="14.25" customHeight="1"/>
-    <row r="413" ht="14.25" customHeight="1"/>
-    <row r="414" ht="14.25" customHeight="1"/>
-    <row r="415" ht="14.25" customHeight="1"/>
-    <row r="416" ht="14.25" customHeight="1"/>
-    <row r="417" ht="14.25" customHeight="1"/>
-    <row r="418" ht="14.25" customHeight="1"/>
-    <row r="419" ht="14.25" customHeight="1"/>
-    <row r="420" ht="14.25" customHeight="1"/>
-    <row r="421" ht="14.25" customHeight="1"/>
-    <row r="422" ht="14.25" customHeight="1"/>
-    <row r="423" ht="14.25" customHeight="1"/>
-    <row r="424" ht="14.25" customHeight="1"/>
-    <row r="425" ht="14.25" customHeight="1"/>
-    <row r="426" ht="14.25" customHeight="1"/>
-    <row r="427" ht="14.25" customHeight="1"/>
-    <row r="428" ht="14.25" customHeight="1"/>
-    <row r="429" ht="14.25" customHeight="1"/>
-    <row r="430" ht="14.25" customHeight="1"/>
-    <row r="431" ht="14.25" customHeight="1"/>
-    <row r="432" ht="14.25" customHeight="1"/>
-    <row r="433" ht="14.25" customHeight="1"/>
-    <row r="434" ht="14.25" customHeight="1"/>
-    <row r="435" ht="14.25" customHeight="1"/>
-    <row r="436" ht="14.25" customHeight="1"/>
-    <row r="437" ht="14.25" customHeight="1"/>
-    <row r="438" ht="14.25" customHeight="1"/>
-    <row r="439" ht="14.25" customHeight="1"/>
-    <row r="440" ht="14.25" customHeight="1"/>
-    <row r="441" ht="14.25" customHeight="1"/>
-    <row r="442" ht="14.25" customHeight="1"/>
-    <row r="443" ht="14.25" customHeight="1"/>
-    <row r="444" ht="14.25" customHeight="1"/>
-    <row r="445" ht="14.25" customHeight="1"/>
-    <row r="446" ht="14.25" customHeight="1"/>
-    <row r="447" ht="14.25" customHeight="1"/>
-    <row r="448" ht="14.25" customHeight="1"/>
-    <row r="449" ht="14.25" customHeight="1"/>
-    <row r="450" ht="14.25" customHeight="1"/>
-    <row r="451" ht="14.25" customHeight="1"/>
-    <row r="452" ht="14.25" customHeight="1"/>
-    <row r="453" ht="14.25" customHeight="1"/>
-    <row r="454" ht="14.25" customHeight="1"/>
-    <row r="455" ht="14.25" customHeight="1"/>
-    <row r="456" ht="14.25" customHeight="1"/>
-    <row r="457" ht="14.25" customHeight="1"/>
-    <row r="458" ht="14.25" customHeight="1"/>
-    <row r="459" ht="14.25" customHeight="1"/>
-    <row r="460" ht="14.25" customHeight="1"/>
-    <row r="461" ht="14.25" customHeight="1"/>
-    <row r="462" ht="14.25" customHeight="1"/>
-    <row r="463" ht="14.25" customHeight="1"/>
-    <row r="464" ht="14.25" customHeight="1"/>
-    <row r="465" ht="14.25" customHeight="1"/>
-    <row r="466" ht="14.25" customHeight="1"/>
-    <row r="467" ht="14.25" customHeight="1"/>
-    <row r="468" ht="14.25" customHeight="1"/>
-    <row r="469" ht="14.25" customHeight="1"/>
-    <row r="470" ht="14.25" customHeight="1"/>
-    <row r="471" ht="14.25" customHeight="1"/>
-    <row r="472" ht="14.25" customHeight="1"/>
-    <row r="473" ht="14.25" customHeight="1"/>
-    <row r="474" ht="14.25" customHeight="1"/>
-    <row r="475" ht="14.25" customHeight="1"/>
-    <row r="476" ht="14.25" customHeight="1"/>
-    <row r="477" ht="14.25" customHeight="1"/>
-    <row r="478" ht="14.25" customHeight="1"/>
-    <row r="479" ht="14.25" customHeight="1"/>
-    <row r="480" ht="14.25" customHeight="1"/>
-    <row r="481" ht="14.25" customHeight="1"/>
-    <row r="482" ht="14.25" customHeight="1"/>
-    <row r="483" ht="14.25" customHeight="1"/>
-    <row r="484" ht="14.25" customHeight="1"/>
-    <row r="485" ht="14.25" customHeight="1"/>
-    <row r="486" ht="14.25" customHeight="1"/>
-    <row r="487" ht="14.25" customHeight="1"/>
-    <row r="488" ht="14.25" customHeight="1"/>
-    <row r="489" ht="14.25" customHeight="1"/>
-    <row r="490" ht="14.25" customHeight="1"/>
-    <row r="491" ht="14.25" customHeight="1"/>
-    <row r="492" ht="14.25" customHeight="1"/>
-    <row r="493" ht="14.25" customHeight="1"/>
-    <row r="494" ht="14.25" customHeight="1"/>
-    <row r="495" ht="14.25" customHeight="1"/>
-    <row r="496" ht="14.25" customHeight="1"/>
-    <row r="497" ht="14.25" customHeight="1"/>
-    <row r="498" ht="14.25" customHeight="1"/>
-    <row r="499" ht="14.25" customHeight="1"/>
-    <row r="500" ht="14.25" customHeight="1"/>
-    <row r="501" ht="14.25" customHeight="1"/>
-    <row r="502" ht="14.25" customHeight="1"/>
-    <row r="503" ht="14.25" customHeight="1"/>
-    <row r="504" ht="14.25" customHeight="1"/>
-    <row r="505" ht="14.25" customHeight="1"/>
-    <row r="506" ht="14.25" customHeight="1"/>
-    <row r="507" ht="14.25" customHeight="1"/>
-    <row r="508" ht="14.25" customHeight="1"/>
-    <row r="509" ht="14.25" customHeight="1"/>
-    <row r="510" ht="14.25" customHeight="1"/>
-    <row r="511" ht="14.25" customHeight="1"/>
-    <row r="512" ht="14.25" customHeight="1"/>
-    <row r="513" ht="14.25" customHeight="1"/>
-    <row r="514" ht="14.25" customHeight="1"/>
-    <row r="515" ht="14.25" customHeight="1"/>
-    <row r="516" ht="14.25" customHeight="1"/>
-    <row r="517" ht="14.25" customHeight="1"/>
-    <row r="518" ht="14.25" customHeight="1"/>
-    <row r="519" ht="14.25" customHeight="1"/>
-    <row r="520" ht="14.25" customHeight="1"/>
-    <row r="521" ht="14.25" customHeight="1"/>
-    <row r="522" ht="14.25" customHeight="1"/>
-    <row r="523" ht="14.25" customHeight="1"/>
-    <row r="524" ht="14.25" customHeight="1"/>
-    <row r="525" ht="14.25" customHeight="1"/>
-    <row r="526" ht="14.25" customHeight="1"/>
-    <row r="527" ht="14.25" customHeight="1"/>
-    <row r="528" ht="14.25" customHeight="1"/>
-    <row r="529" ht="14.25" customHeight="1"/>
-    <row r="530" ht="14.25" customHeight="1"/>
-    <row r="531" ht="14.25" customHeight="1"/>
-    <row r="532" ht="14.25" customHeight="1"/>
-    <row r="533" ht="14.25" customHeight="1"/>
-    <row r="534" ht="14.25" customHeight="1"/>
-    <row r="535" ht="14.25" customHeight="1"/>
-    <row r="536" ht="14.25" customHeight="1"/>
-    <row r="537" ht="14.25" customHeight="1"/>
-    <row r="538" ht="14.25" customHeight="1"/>
-    <row r="539" ht="14.25" customHeight="1"/>
-    <row r="540" ht="14.25" customHeight="1"/>
-    <row r="541" ht="14.25" customHeight="1"/>
-    <row r="542" ht="14.25" customHeight="1"/>
-    <row r="543" ht="14.25" customHeight="1"/>
-    <row r="544" ht="14.25" customHeight="1"/>
-    <row r="545" ht="14.25" customHeight="1"/>
-    <row r="546" ht="14.25" customHeight="1"/>
-    <row r="547" ht="14.25" customHeight="1"/>
-    <row r="548" ht="14.25" customHeight="1"/>
-    <row r="549" ht="14.25" customHeight="1"/>
-    <row r="550" ht="14.25" customHeight="1"/>
-    <row r="551" ht="14.25" customHeight="1"/>
-    <row r="552" ht="14.25" customHeight="1"/>
-    <row r="553" ht="14.25" customHeight="1"/>
-    <row r="554" ht="14.25" customHeight="1"/>
-    <row r="555" ht="14.25" customHeight="1"/>
-    <row r="556" ht="14.25" customHeight="1"/>
-    <row r="557" ht="14.25" customHeight="1"/>
-    <row r="558" ht="14.25" customHeight="1"/>
-    <row r="559" ht="14.25" customHeight="1"/>
-    <row r="560" ht="14.25" customHeight="1"/>
-    <row r="561" ht="14.25" customHeight="1"/>
-    <row r="562" ht="14.25" customHeight="1"/>
-    <row r="563" ht="14.25" customHeight="1"/>
-    <row r="564" ht="14.25" customHeight="1"/>
-    <row r="565" ht="14.25" customHeight="1"/>
-    <row r="566" ht="14.25" customHeight="1"/>
-    <row r="567" ht="14.25" customHeight="1"/>
-    <row r="568" ht="14.25" customHeight="1"/>
-    <row r="569" ht="14.25" customHeight="1"/>
-    <row r="570" ht="14.25" customHeight="1"/>
-    <row r="571" ht="14.25" customHeight="1"/>
-    <row r="572" ht="14.25" customHeight="1"/>
-    <row r="573" ht="14.25" customHeight="1"/>
-    <row r="574" ht="14.25" customHeight="1"/>
-    <row r="575" ht="14.25" customHeight="1"/>
-    <row r="576" ht="14.25" customHeight="1"/>
-    <row r="577" ht="14.25" customHeight="1"/>
-    <row r="578" ht="14.25" customHeight="1"/>
-    <row r="579" ht="14.25" customHeight="1"/>
-    <row r="580" ht="14.25" customHeight="1"/>
-    <row r="581" ht="14.25" customHeight="1"/>
-    <row r="582" ht="14.25" customHeight="1"/>
-    <row r="583" ht="14.25" customHeight="1"/>
-    <row r="584" ht="14.25" customHeight="1"/>
-    <row r="585" ht="14.25" customHeight="1"/>
-    <row r="586" ht="14.25" customHeight="1"/>
-    <row r="587" ht="14.25" customHeight="1"/>
-    <row r="588" ht="14.25" customHeight="1"/>
-    <row r="589" ht="14.25" customHeight="1"/>
-    <row r="590" ht="14.25" customHeight="1"/>
-    <row r="591" ht="14.25" customHeight="1"/>
-    <row r="592" ht="14.25" customHeight="1"/>
-    <row r="593" ht="14.25" customHeight="1"/>
-    <row r="594" ht="14.25" customHeight="1"/>
-    <row r="595" ht="14.25" customHeight="1"/>
-    <row r="596" ht="14.25" customHeight="1"/>
-    <row r="597" ht="14.25" customHeight="1"/>
-    <row r="598" ht="14.25" customHeight="1"/>
-    <row r="599" ht="14.25" customHeight="1"/>
-    <row r="600" ht="14.25" customHeight="1"/>
-    <row r="601" ht="14.25" customHeight="1"/>
-    <row r="602" ht="14.25" customHeight="1"/>
-    <row r="603" ht="14.25" customHeight="1"/>
-    <row r="604" ht="14.25" customHeight="1"/>
-    <row r="605" ht="14.25" customHeight="1"/>
-    <row r="606" ht="14.25" customHeight="1"/>
-    <row r="607" ht="14.25" customHeight="1"/>
-    <row r="608" ht="14.25" customHeight="1"/>
-    <row r="609" ht="14.25" customHeight="1"/>
-    <row r="610" ht="14.25" customHeight="1"/>
-    <row r="611" ht="14.25" customHeight="1"/>
-    <row r="612" ht="14.25" customHeight="1"/>
-    <row r="613" ht="14.25" customHeight="1"/>
-    <row r="614" ht="14.25" customHeight="1"/>
-    <row r="615" ht="14.25" customHeight="1"/>
-    <row r="616" ht="14.25" customHeight="1"/>
-    <row r="617" ht="14.25" customHeight="1"/>
-    <row r="618" ht="14.25" customHeight="1"/>
-    <row r="619" ht="14.25" customHeight="1"/>
-    <row r="620" ht="14.25" customHeight="1"/>
-    <row r="621" ht="14.25" customHeight="1"/>
-    <row r="622" ht="14.25" customHeight="1"/>
-    <row r="623" ht="14.25" customHeight="1"/>
-    <row r="624" ht="14.25" customHeight="1"/>
-    <row r="625" ht="14.25" customHeight="1"/>
-    <row r="626" ht="14.25" customHeight="1"/>
-    <row r="627" ht="14.25" customHeight="1"/>
-    <row r="628" ht="14.25" customHeight="1"/>
-    <row r="629" ht="14.25" customHeight="1"/>
-    <row r="630" ht="14.25" customHeight="1"/>
-    <row r="631" ht="14.25" customHeight="1"/>
-    <row r="632" ht="14.25" customHeight="1"/>
-    <row r="633" ht="14.25" customHeight="1"/>
-    <row r="634" ht="14.25" customHeight="1"/>
-    <row r="635" ht="14.25" customHeight="1"/>
-    <row r="636" ht="14.25" customHeight="1"/>
-    <row r="637" ht="14.25" customHeight="1"/>
-    <row r="638" ht="14.25" customHeight="1"/>
-    <row r="639" ht="14.25" customHeight="1"/>
-    <row r="640" ht="14.25" customHeight="1"/>
-    <row r="641" ht="14.25" customHeight="1"/>
-    <row r="642" ht="14.25" customHeight="1"/>
-    <row r="643" ht="14.25" customHeight="1"/>
-    <row r="644" ht="14.25" customHeight="1"/>
-    <row r="645" ht="14.25" customHeight="1"/>
-    <row r="646" ht="14.25" customHeight="1"/>
-    <row r="647" ht="14.25" customHeight="1"/>
-    <row r="648" ht="14.25" customHeight="1"/>
-    <row r="649" ht="14.25" customHeight="1"/>
-    <row r="650" ht="14.25" customHeight="1"/>
-    <row r="651" ht="14.25" customHeight="1"/>
-    <row r="652" ht="14.25" customHeight="1"/>
-    <row r="653" ht="14.25" customHeight="1"/>
-    <row r="654" ht="14.25" customHeight="1"/>
-    <row r="655" ht="14.25" customHeight="1"/>
-    <row r="656" ht="14.25" customHeight="1"/>
-    <row r="657" ht="14.25" customHeight="1"/>
-    <row r="658" ht="14.25" customHeight="1"/>
-    <row r="659" ht="14.25" customHeight="1"/>
-    <row r="660" ht="14.25" customHeight="1"/>
-    <row r="661" ht="14.25" customHeight="1"/>
-    <row r="662" ht="14.25" customHeight="1"/>
-    <row r="663" ht="14.25" customHeight="1"/>
-    <row r="664" ht="14.25" customHeight="1"/>
-    <row r="665" ht="14.25" customHeight="1"/>
-    <row r="666" ht="14.25" customHeight="1"/>
-    <row r="667" ht="14.25" customHeight="1"/>
-    <row r="668" ht="14.25" customHeight="1"/>
-    <row r="669" ht="14.25" customHeight="1"/>
-    <row r="670" ht="14.25" customHeight="1"/>
-    <row r="671" ht="14.25" customHeight="1"/>
-    <row r="672" ht="14.25" customHeight="1"/>
-    <row r="673" ht="14.25" customHeight="1"/>
-    <row r="674" ht="14.25" customHeight="1"/>
-    <row r="675" ht="14.25" customHeight="1"/>
-    <row r="676" ht="14.25" customHeight="1"/>
-    <row r="677" ht="14.25" customHeight="1"/>
-    <row r="678" ht="14.25" customHeight="1"/>
-    <row r="679" ht="14.25" customHeight="1"/>
-    <row r="680" ht="14.25" customHeight="1"/>
-    <row r="681" ht="14.25" customHeight="1"/>
-    <row r="682" ht="14.25" customHeight="1"/>
-    <row r="683" ht="14.25" customHeight="1"/>
-    <row r="684" ht="14.25" customHeight="1"/>
-    <row r="685" ht="14.25" customHeight="1"/>
-    <row r="686" ht="14.25" customHeight="1"/>
-    <row r="687" ht="14.25" customHeight="1"/>
-    <row r="688" ht="14.25" customHeight="1"/>
-    <row r="689" ht="14.25" customHeight="1"/>
-    <row r="690" ht="14.25" customHeight="1"/>
-    <row r="691" ht="14.25" customHeight="1"/>
-    <row r="692" ht="14.25" customHeight="1"/>
-    <row r="693" ht="14.25" customHeight="1"/>
-    <row r="694" ht="14.25" customHeight="1"/>
-    <row r="695" ht="14.25" customHeight="1"/>
-    <row r="696" ht="14.25" customHeight="1"/>
-    <row r="697" ht="14.25" customHeight="1"/>
-    <row r="698" ht="14.25" customHeight="1"/>
-    <row r="699" ht="14.25" customHeight="1"/>
-    <row r="700" ht="14.25" customHeight="1"/>
-    <row r="701" ht="14.25" customHeight="1"/>
-    <row r="702" ht="14.25" customHeight="1"/>
-    <row r="703" ht="14.25" customHeight="1"/>
-    <row r="704" ht="14.25" customHeight="1"/>
-    <row r="705" ht="14.25" customHeight="1"/>
-    <row r="706" ht="14.25" customHeight="1"/>
-    <row r="707" ht="14.25" customHeight="1"/>
-    <row r="708" ht="14.25" customHeight="1"/>
-    <row r="709" ht="14.25" customHeight="1"/>
-    <row r="710" ht="14.25" customHeight="1"/>
-    <row r="711" ht="14.25" customHeight="1"/>
-    <row r="712" ht="14.25" customHeight="1"/>
-    <row r="713" ht="14.25" customHeight="1"/>
-    <row r="714" ht="14.25" customHeight="1"/>
-    <row r="715" ht="14.25" customHeight="1"/>
-    <row r="716" ht="14.25" customHeight="1"/>
-    <row r="717" ht="14.25" customHeight="1"/>
-    <row r="718" ht="14.25" customHeight="1"/>
-    <row r="719" ht="14.25" customHeight="1"/>
-    <row r="720" ht="14.25" customHeight="1"/>
-    <row r="721" ht="14.25" customHeight="1"/>
-    <row r="722" ht="14.25" customHeight="1"/>
-    <row r="723" ht="14.25" customHeight="1"/>
-    <row r="724" ht="14.25" customHeight="1"/>
-    <row r="725" ht="14.25" customHeight="1"/>
-    <row r="726" ht="14.25" customHeight="1"/>
-    <row r="727" ht="14.25" customHeight="1"/>
-    <row r="728" ht="14.25" customHeight="1"/>
-    <row r="729" ht="14.25" customHeight="1"/>
-    <row r="730" ht="14.25" customHeight="1"/>
-    <row r="731" ht="14.25" customHeight="1"/>
-    <row r="732" ht="14.25" customHeight="1"/>
-    <row r="733" ht="14.25" customHeight="1"/>
-    <row r="734" ht="14.25" customHeight="1"/>
-    <row r="735" ht="14.25" customHeight="1"/>
-    <row r="736" ht="14.25" customHeight="1"/>
-    <row r="737" ht="14.25" customHeight="1"/>
-    <row r="738" ht="14.25" customHeight="1"/>
-    <row r="739" ht="14.25" customHeight="1"/>
-    <row r="740" ht="14.25" customHeight="1"/>
-    <row r="741" ht="14.25" customHeight="1"/>
-    <row r="742" ht="14.25" customHeight="1"/>
-    <row r="743" ht="14.25" customHeight="1"/>
-    <row r="744" ht="14.25" customHeight="1"/>
-    <row r="745" ht="14.25" customHeight="1"/>
-    <row r="746" ht="14.25" customHeight="1"/>
-    <row r="747" ht="14.25" customHeight="1"/>
-    <row r="748" ht="14.25" customHeight="1"/>
-    <row r="749" ht="14.25" customHeight="1"/>
-    <row r="750" ht="14.25" customHeight="1"/>
-    <row r="751" ht="14.25" customHeight="1"/>
-    <row r="752" ht="14.25" customHeight="1"/>
-    <row r="753" ht="14.25" customHeight="1"/>
-    <row r="754" ht="14.25" customHeight="1"/>
-    <row r="755" ht="14.25" customHeight="1"/>
-    <row r="756" ht="14.25" customHeight="1"/>
-    <row r="757" ht="14.25" customHeight="1"/>
-    <row r="758" ht="14.25" customHeight="1"/>
-    <row r="759" ht="14.25" customHeight="1"/>
-    <row r="760" ht="14.25" customHeight="1"/>
-    <row r="761" ht="14.25" customHeight="1"/>
-    <row r="762" ht="14.25" customHeight="1"/>
-    <row r="763" ht="14.25" customHeight="1"/>
-    <row r="764" ht="14.25" customHeight="1"/>
-    <row r="765" ht="14.25" customHeight="1"/>
-    <row r="766" ht="14.25" customHeight="1"/>
-    <row r="767" ht="14.25" customHeight="1"/>
-    <row r="768" ht="14.25" customHeight="1"/>
-    <row r="769" ht="14.25" customHeight="1"/>
-    <row r="770" ht="14.25" customHeight="1"/>
-    <row r="771" ht="14.25" customHeight="1"/>
-    <row r="772" ht="14.25" customHeight="1"/>
-    <row r="773" ht="14.25" customHeight="1"/>
-    <row r="774" ht="14.25" customHeight="1"/>
-    <row r="775" ht="14.25" customHeight="1"/>
-    <row r="776" ht="14.25" customHeight="1"/>
-    <row r="777" ht="14.25" customHeight="1"/>
-    <row r="778" ht="14.25" customHeight="1"/>
-    <row r="779" ht="14.25" customHeight="1"/>
-    <row r="780" ht="14.25" customHeight="1"/>
-    <row r="781" ht="14.25" customHeight="1"/>
-    <row r="782" ht="14.25" customHeight="1"/>
-    <row r="783" ht="14.25" customHeight="1"/>
-    <row r="784" ht="14.25" customHeight="1"/>
-    <row r="785" ht="14.25" customHeight="1"/>
-    <row r="786" ht="14.25" customHeight="1"/>
-    <row r="787" ht="14.25" customHeight="1"/>
-    <row r="788" ht="14.25" customHeight="1"/>
-    <row r="789" ht="14.25" customHeight="1"/>
-    <row r="790" ht="14.25" customHeight="1"/>
-    <row r="791" ht="14.25" customHeight="1"/>
-    <row r="792" ht="14.25" customHeight="1"/>
-    <row r="793" ht="14.25" customHeight="1"/>
-    <row r="794" ht="14.25" customHeight="1"/>
-    <row r="795" ht="14.25" customHeight="1"/>
-    <row r="796" ht="14.25" customHeight="1"/>
-    <row r="797" ht="14.25" customHeight="1"/>
-    <row r="798" ht="14.25" customHeight="1"/>
-    <row r="799" ht="14.25" customHeight="1"/>
-    <row r="800" ht="14.25" customHeight="1"/>
-    <row r="801" ht="14.25" customHeight="1"/>
-    <row r="802" ht="14.25" customHeight="1"/>
-    <row r="803" ht="14.25" customHeight="1"/>
-    <row r="804" ht="14.25" customHeight="1"/>
-    <row r="805" ht="14.25" customHeight="1"/>
-    <row r="806" ht="14.25" customHeight="1"/>
-    <row r="807" ht="14.25" customHeight="1"/>
-    <row r="808" ht="14.25" customHeight="1"/>
-    <row r="809" ht="14.25" customHeight="1"/>
-    <row r="810" ht="14.25" customHeight="1"/>
-    <row r="811" ht="14.25" customHeight="1"/>
-    <row r="812" ht="14.25" customHeight="1"/>
-    <row r="813" ht="14.25" customHeight="1"/>
-    <row r="814" ht="14.25" customHeight="1"/>
-    <row r="815" ht="14.25" customHeight="1"/>
-    <row r="816" ht="14.25" customHeight="1"/>
-    <row r="817" ht="14.25" customHeight="1"/>
-    <row r="818" ht="14.25" customHeight="1"/>
-    <row r="819" ht="14.25" customHeight="1"/>
-    <row r="820" ht="14.25" customHeight="1"/>
-    <row r="821" ht="14.25" customHeight="1"/>
-    <row r="822" ht="14.25" customHeight="1"/>
-    <row r="823" ht="14.25" customHeight="1"/>
-    <row r="824" ht="14.25" customHeight="1"/>
-    <row r="825" ht="14.25" customHeight="1"/>
-    <row r="826" ht="14.25" customHeight="1"/>
-    <row r="827" ht="14.25" customHeight="1"/>
-    <row r="828" ht="14.25" customHeight="1"/>
-    <row r="829" ht="14.25" customHeight="1"/>
-    <row r="830" ht="14.25" customHeight="1"/>
-    <row r="831" ht="14.25" customHeight="1"/>
-    <row r="832" ht="14.25" customHeight="1"/>
-    <row r="833" ht="14.25" customHeight="1"/>
-    <row r="834" ht="14.25" customHeight="1"/>
-    <row r="835" ht="14.25" customHeight="1"/>
-    <row r="836" ht="14.25" customHeight="1"/>
-    <row r="837" ht="14.25" customHeight="1"/>
-    <row r="838" ht="14.25" customHeight="1"/>
-    <row r="839" ht="14.25" customHeight="1"/>
-    <row r="840" ht="14.25" customHeight="1"/>
-    <row r="841" ht="14.25" customHeight="1"/>
-    <row r="842" ht="14.25" customHeight="1"/>
-    <row r="843" ht="14.25" customHeight="1"/>
-    <row r="844" ht="14.25" customHeight="1"/>
-    <row r="845" ht="14.25" customHeight="1"/>
-    <row r="846" ht="14.25" customHeight="1"/>
-    <row r="847" ht="14.25" customHeight="1"/>
-    <row r="848" ht="14.25" customHeight="1"/>
-    <row r="849" ht="14.25" customHeight="1"/>
-    <row r="850" ht="14.25" customHeight="1"/>
-    <row r="851" ht="14.25" customHeight="1"/>
-    <row r="852" ht="14.25" customHeight="1"/>
-    <row r="853" ht="14.25" customHeight="1"/>
-    <row r="854" ht="14.25" customHeight="1"/>
-    <row r="855" ht="14.25" customHeight="1"/>
-    <row r="856" ht="14.25" customHeight="1"/>
-    <row r="857" ht="14.25" customHeight="1"/>
-    <row r="858" ht="14.25" customHeight="1"/>
-    <row r="859" ht="14.25" customHeight="1"/>
-    <row r="860" ht="14.25" customHeight="1"/>
-    <row r="861" ht="14.25" customHeight="1"/>
-    <row r="862" ht="14.25" customHeight="1"/>
-    <row r="863" ht="14.25" customHeight="1"/>
-    <row r="864" ht="14.25" customHeight="1"/>
-    <row r="865" ht="14.25" customHeight="1"/>
-    <row r="866" ht="14.25" customHeight="1"/>
-    <row r="867" ht="14.25" customHeight="1"/>
-    <row r="868" ht="14.25" customHeight="1"/>
-    <row r="869" ht="14.25" customHeight="1"/>
-    <row r="870" ht="14.25" customHeight="1"/>
-    <row r="871" ht="14.25" customHeight="1"/>
-    <row r="872" ht="14.25" customHeight="1"/>
-    <row r="873" ht="14.25" customHeight="1"/>
-    <row r="874" ht="14.25" customHeight="1"/>
-    <row r="875" ht="14.25" customHeight="1"/>
-    <row r="876" ht="14.25" customHeight="1"/>
-    <row r="877" ht="14.25" customHeight="1"/>
-    <row r="878" ht="14.25" customHeight="1"/>
-    <row r="879" ht="14.25" customHeight="1"/>
-    <row r="880" ht="14.25" customHeight="1"/>
-    <row r="881" ht="14.25" customHeight="1"/>
-    <row r="882" ht="14.25" customHeight="1"/>
-    <row r="883" ht="14.25" customHeight="1"/>
-    <row r="884" ht="14.25" customHeight="1"/>
-    <row r="885" ht="14.25" customHeight="1"/>
-    <row r="886" ht="14.25" customHeight="1"/>
-    <row r="887" ht="14.25" customHeight="1"/>
-    <row r="888" ht="14.25" customHeight="1"/>
-    <row r="889" ht="14.25" customHeight="1"/>
-    <row r="890" ht="14.25" customHeight="1"/>
-    <row r="891" ht="14.25" customHeight="1"/>
-    <row r="892" ht="14.25" customHeight="1"/>
-    <row r="893" ht="14.25" customHeight="1"/>
-    <row r="894" ht="14.25" customHeight="1"/>
-    <row r="895" ht="14.25" customHeight="1"/>
-    <row r="896" ht="14.25" customHeight="1"/>
-    <row r="897" ht="14.25" customHeight="1"/>
-    <row r="898" ht="14.25" customHeight="1"/>
-    <row r="899" ht="14.25" customHeight="1"/>
-    <row r="900" ht="14.25" customHeight="1"/>
-    <row r="901" ht="14.25" customHeight="1"/>
-    <row r="902" ht="14.25" customHeight="1"/>
-    <row r="903" ht="14.25" customHeight="1"/>
-    <row r="904" ht="14.25" customHeight="1"/>
-    <row r="905" ht="14.25" customHeight="1"/>
-    <row r="906" ht="14.25" customHeight="1"/>
-    <row r="907" ht="14.25" customHeight="1"/>
-    <row r="908" ht="14.25" customHeight="1"/>
-    <row r="909" ht="14.25" customHeight="1"/>
-    <row r="910" ht="14.25" customHeight="1"/>
-    <row r="911" ht="14.25" customHeight="1"/>
-    <row r="912" ht="14.25" customHeight="1"/>
-    <row r="913" ht="14.25" customHeight="1"/>
-    <row r="914" ht="14.25" customHeight="1"/>
-    <row r="915" ht="14.25" customHeight="1"/>
-    <row r="916" ht="14.25" customHeight="1"/>
-    <row r="917" ht="14.25" customHeight="1"/>
-    <row r="918" ht="14.25" customHeight="1"/>
-    <row r="919" ht="14.25" customHeight="1"/>
-    <row r="920" ht="14.25" customHeight="1"/>
-    <row r="921" ht="14.25" customHeight="1"/>
-    <row r="922" ht="14.25" customHeight="1"/>
-    <row r="923" ht="14.25" customHeight="1"/>
-    <row r="924" ht="14.25" customHeight="1"/>
-    <row r="925" ht="14.25" customHeight="1"/>
-    <row r="926" ht="14.25" customHeight="1"/>
-    <row r="927" ht="14.25" customHeight="1"/>
-    <row r="928" ht="14.25" customHeight="1"/>
-    <row r="929" ht="14.25" customHeight="1"/>
-    <row r="930" ht="14.25" customHeight="1"/>
-    <row r="931" ht="14.25" customHeight="1"/>
-    <row r="932" ht="14.25" customHeight="1"/>
-    <row r="933" ht="14.25" customHeight="1"/>
-    <row r="934" ht="14.25" customHeight="1"/>
-    <row r="935" ht="14.25" customHeight="1"/>
-    <row r="936" ht="14.25" customHeight="1"/>
-    <row r="937" ht="14.25" customHeight="1"/>
-    <row r="938" ht="14.25" customHeight="1"/>
-    <row r="939" ht="14.25" customHeight="1"/>
-    <row r="940" ht="14.25" customHeight="1"/>
-    <row r="941" ht="14.25" customHeight="1"/>
-    <row r="942" ht="14.25" customHeight="1"/>
-    <row r="943" ht="14.25" customHeight="1"/>
-    <row r="944" ht="14.25" customHeight="1"/>
-    <row r="945" ht="14.25" customHeight="1"/>
-    <row r="946" ht="14.25" customHeight="1"/>
-    <row r="947" ht="14.25" customHeight="1"/>
-    <row r="948" ht="14.25" customHeight="1"/>
-    <row r="949" ht="14.25" customHeight="1"/>
-    <row r="950" ht="14.25" customHeight="1"/>
-    <row r="951" ht="14.25" customHeight="1"/>
-    <row r="952" ht="14.25" customHeight="1"/>
-    <row r="953" ht="14.25" customHeight="1"/>
-    <row r="954" ht="14.25" customHeight="1"/>
-    <row r="955" ht="14.25" customHeight="1"/>
-    <row r="956" ht="14.25" customHeight="1"/>
-    <row r="957" ht="14.25" customHeight="1"/>
-    <row r="958" ht="14.25" customHeight="1"/>
-    <row r="959" ht="14.25" customHeight="1"/>
-    <row r="960" ht="14.25" customHeight="1"/>
-    <row r="961" ht="14.25" customHeight="1"/>
-    <row r="962" ht="14.25" customHeight="1"/>
-    <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
-    <row r="973" ht="14.25" customHeight="1"/>
-    <row r="974" ht="14.25" customHeight="1"/>
-    <row r="975" ht="14.25" customHeight="1"/>
-    <row r="976" ht="14.25" customHeight="1"/>
-    <row r="977" ht="14.25" customHeight="1"/>
-    <row r="978" ht="14.25" customHeight="1"/>
-    <row r="979" ht="14.25" customHeight="1"/>
-    <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
-    <row r="1001" ht="14.25" customHeight="1"/>
-    <row r="1002" ht="14.25" customHeight="1"/>
-    <row r="1003" ht="14.25" customHeight="1"/>
-    <row r="1004" ht="14.25" customHeight="1"/>
-    <row r="1005" ht="14.25" customHeight="1"/>
-    <row r="1006" ht="14.25" customHeight="1"/>
-    <row r="1007" ht="14.25" customHeight="1"/>
-    <row r="1008" ht="14.25" customHeight="1"/>
-    <row r="1009" ht="14.25" customHeight="1"/>
-    <row r="1010" ht="14.25" customHeight="1"/>
-    <row r="1011" ht="14.25" customHeight="1"/>
-    <row r="1012" ht="14.25" customHeight="1"/>
-    <row r="1013" ht="14.25" customHeight="1"/>
-    <row r="1014" ht="14.25" customHeight="1"/>
-    <row r="1015" ht="14.25" customHeight="1"/>
-    <row r="1016" ht="14.25" customHeight="1"/>
-    <row r="1017" ht="14.25" customHeight="1"/>
-    <row r="1018" ht="14.25" customHeight="1"/>
-    <row r="1019" ht="14.25" customHeight="1"/>
-    <row r="1020" ht="14.25" customHeight="1"/>
-    <row r="1021" ht="14.25" customHeight="1"/>
-    <row r="1022" ht="14.25" customHeight="1"/>
-    <row r="1023" ht="14.25" customHeight="1"/>
-    <row r="1024" ht="14.25" customHeight="1"/>
-    <row r="1025" ht="14.25" customHeight="1"/>
-    <row r="1026" ht="14.25" customHeight="1"/>
-    <row r="1027" ht="14.25" customHeight="1"/>
-    <row r="1028" ht="14.25" customHeight="1"/>
-    <row r="1029" ht="14.25" customHeight="1"/>
-    <row r="1030" ht="14.25" customHeight="1"/>
-    <row r="1031" ht="14.25" customHeight="1"/>
-    <row r="1032" ht="14.25" customHeight="1"/>
-    <row r="1033" ht="14.25" customHeight="1"/>
-    <row r="1034" ht="14.25" customHeight="1"/>
-    <row r="1035" ht="14.25" customHeight="1"/>
-    <row r="1036" ht="14.25" customHeight="1"/>
-    <row r="1037" ht="14.25" customHeight="1"/>
-    <row r="1038" ht="14.25" customHeight="1"/>
-    <row r="1039" ht="14.25" customHeight="1"/>
-    <row r="1040" ht="14.25" customHeight="1"/>
-    <row r="1041" ht="14.25" customHeight="1"/>
-    <row r="1042" ht="14.25" customHeight="1"/>
-    <row r="1043" ht="14.25" customHeight="1"/>
-    <row r="1044" ht="14.25" customHeight="1"/>
-    <row r="1045" ht="14.25" customHeight="1"/>
-    <row r="1046" ht="14.25" customHeight="1"/>
-    <row r="1047" ht="14.25" customHeight="1"/>
-    <row r="1048" ht="14.25" customHeight="1"/>
-    <row r="1049" ht="14.25" customHeight="1"/>
-    <row r="1050" ht="14.25" customHeight="1"/>
-    <row r="1051" ht="14.25" customHeight="1"/>
-    <row r="1052" ht="14.25" customHeight="1"/>
-    <row r="1053" ht="14.25" customHeight="1"/>
-    <row r="1054" ht="14.25" customHeight="1"/>
-    <row r="1055" ht="14.25" customHeight="1"/>
-    <row r="1056" ht="14.25" customHeight="1"/>
-    <row r="1057" ht="14.25" customHeight="1"/>
-    <row r="1058" ht="14.25" customHeight="1"/>
-    <row r="1059" ht="14.25" customHeight="1"/>
-    <row r="1060" ht="14.25" customHeight="1"/>
-    <row r="1061" ht="14.25" customHeight="1"/>
-    <row r="1062" ht="14.25" customHeight="1"/>
-    <row r="1063" ht="14.25" customHeight="1"/>
-    <row r="1064" ht="14.25" customHeight="1"/>
-    <row r="1065" ht="14.25" customHeight="1"/>
-    <row r="1066" ht="14.25" customHeight="1"/>
-    <row r="1067" ht="14.25" customHeight="1"/>
-    <row r="1068" ht="14.25" customHeight="1"/>
-    <row r="1069" ht="14.25" customHeight="1"/>
-    <row r="1070" ht="14.25" customHeight="1"/>
-    <row r="1071" ht="14.25" customHeight="1"/>
-    <row r="1072" ht="14.25" customHeight="1"/>
-    <row r="1073" ht="14.25" customHeight="1"/>
-    <row r="1074" ht="14.25" customHeight="1"/>
-    <row r="1075" ht="14.25" customHeight="1"/>
-    <row r="1076" ht="14.25" customHeight="1"/>
-    <row r="1077" ht="14.25" customHeight="1"/>
-    <row r="1078" ht="14.25" customHeight="1"/>
-    <row r="1079" ht="14.25" customHeight="1"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Log Messages in WorkFlows
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harih\OneDrive\Documents\UiPath\Invoices\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8874F57-7FD7-4E15-B63A-F7DE3944736B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E5D86E-2EF5-495C-84C5-3E97165A8504}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="506">
   <si>
     <t>Name</t>
   </si>
@@ -1527,6 +1527,21 @@
   </si>
   <si>
     <t>Multiple Line GL Account Entry started</t>
+  </si>
+  <si>
+    <t>LogLinesWindowEntryStart</t>
+  </si>
+  <si>
+    <t>Entering Lines window fields started</t>
+  </si>
+  <si>
+    <t>LogLinesWindowEntrySuccess</t>
+  </si>
+  <si>
+    <t>Entering Lines window fields success</t>
+  </si>
+  <si>
+    <t>TimeOut_IEModeEdgeBrowser</t>
   </si>
 </sst>
 </file>
@@ -1559,18 +1574,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1585,7 +1594,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1609,8 +1618,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
@@ -1927,7 +1934,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1231"/>
+  <dimension ref="A1:Z1226"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="49.54296875" customWidth="1"/>
@@ -2542,7 +2549,7 @@
       <c r="A74" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="B74" s="15" t="s">
+      <c r="B74" s="13" t="s">
         <v>298</v>
       </c>
     </row>
@@ -2550,7 +2557,7 @@
       <c r="A75" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="B75" s="15" t="s">
+      <c r="B75" s="13" t="s">
         <v>299</v>
       </c>
     </row>
@@ -2558,7 +2565,7 @@
       <c r="A76" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="B76" s="15" t="s">
+      <c r="B76" s="13" t="s">
         <v>300</v>
       </c>
     </row>
@@ -2566,7 +2573,7 @@
       <c r="A77" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="B77" s="15" t="s">
+      <c r="B77" s="13" t="s">
         <v>301</v>
       </c>
     </row>
@@ -2574,7 +2581,7 @@
       <c r="A78" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="B78" s="15" t="s">
+      <c r="B78" s="13" t="s">
         <v>302</v>
       </c>
     </row>
@@ -2582,7 +2589,7 @@
       <c r="A79" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="B79" s="15" t="s">
+      <c r="B79" s="13" t="s">
         <v>303</v>
       </c>
     </row>
@@ -2590,7 +2597,7 @@
       <c r="A80" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="B80" s="15" t="s">
+      <c r="B80" s="13" t="s">
         <v>304</v>
       </c>
     </row>
@@ -2598,7 +2605,7 @@
       <c r="A81" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="B81" s="15" t="s">
+      <c r="B81" s="13" t="s">
         <v>305</v>
       </c>
     </row>
@@ -2606,7 +2613,7 @@
       <c r="A82" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="B82" s="15" t="s">
+      <c r="B82" s="13" t="s">
         <v>306</v>
       </c>
     </row>
@@ -2614,7 +2621,7 @@
       <c r="A83" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="B83" s="15" t="s">
+      <c r="B83" s="13" t="s">
         <v>307</v>
       </c>
     </row>
@@ -2622,7 +2629,7 @@
       <c r="A84" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="B84" s="15" t="s">
+      <c r="B84" s="13" t="s">
         <v>308</v>
       </c>
     </row>
@@ -2630,7 +2637,7 @@
       <c r="A85" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="B85" s="15" t="s">
+      <c r="B85" s="13" t="s">
         <v>309</v>
       </c>
     </row>
@@ -2638,7 +2645,7 @@
       <c r="A86" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="B86" s="15" t="s">
+      <c r="B86" s="13" t="s">
         <v>310</v>
       </c>
     </row>
@@ -2646,7 +2653,7 @@
       <c r="A87" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="B87" s="15" t="s">
+      <c r="B87" s="13" t="s">
         <v>311</v>
       </c>
     </row>
@@ -2654,7 +2661,7 @@
       <c r="A88" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="B88" s="15" t="s">
+      <c r="B88" s="13" t="s">
         <v>312</v>
       </c>
     </row>
@@ -2662,7 +2669,7 @@
       <c r="A89" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="B89" s="15" t="s">
+      <c r="B89" s="13" t="s">
         <v>313</v>
       </c>
     </row>
@@ -3111,12 +3118,20 @@
       </c>
     </row>
     <row r="154" spans="1:2" ht="14.5">
-      <c r="A154" s="2"/>
-      <c r="B154" s="9"/>
+      <c r="A154" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="B154" s="9" t="s">
+        <v>502</v>
+      </c>
     </row>
     <row r="155" spans="1:2" ht="14.5">
-      <c r="A155" s="2"/>
-      <c r="B155" s="9"/>
+      <c r="A155" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="B155" s="9" t="s">
+        <v>504</v>
+      </c>
     </row>
     <row r="156" spans="1:2" ht="14.5">
       <c r="A156" s="2"/>
@@ -3126,397 +3141,429 @@
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
     </row>
-    <row r="158" spans="1:2" ht="14.5">
-      <c r="A158" s="2"/>
-      <c r="B158" s="2"/>
-    </row>
-    <row r="159" spans="1:2" ht="14.5">
-      <c r="A159" s="2"/>
-      <c r="B159" s="2"/>
-    </row>
-    <row r="160" spans="1:2" ht="14.5">
-      <c r="A160" s="2"/>
-      <c r="B160" s="2"/>
-    </row>
-    <row r="161" spans="1:3" s="9" customFormat="1" ht="14.5">
-      <c r="A161" s="16"/>
-      <c r="B161" s="16"/>
-    </row>
-    <row r="162" spans="1:3" s="9" customFormat="1" ht="14.5">
-      <c r="A162" s="16"/>
-      <c r="B162" s="16"/>
-    </row>
-    <row r="163" spans="1:3" ht="14.5">
-      <c r="A163" s="2"/>
-      <c r="B163" s="2"/>
-    </row>
-    <row r="164" spans="1:3" s="13" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A164" s="13" t="s">
+    <row r="158" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A158" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B164" s="13" t="s">
+      <c r="B158" s="9" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A165" t="s">
+    <row r="159" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A159" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B159" s="9" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="166" spans="1:3" s="13" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A166" s="13" t="s">
+    <row r="160" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A160" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B166" s="13" t="s">
+      <c r="B160" s="9" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="167" spans="1:3" s="13" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A167" s="13" t="s">
+    <row r="161" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A161" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="B167" s="13" t="s">
+      <c r="B161" s="9" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="168" spans="1:3" s="13" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A168" s="13" t="s">
+    <row r="162" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A162" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B168" s="13" t="s">
+      <c r="B162" s="9" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="169" spans="1:3" s="13" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A169" s="14" t="s">
+    <row r="163" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A163" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="B169" s="14" t="s">
+      <c r="B163" s="14" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="170" spans="1:3" s="13" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A170" s="13" t="s">
+    <row r="164" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A164" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="B170" s="13" t="s">
+      <c r="B164" s="9" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="171" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A171" s="9" t="s">
+    <row r="165" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A165" s="9" t="s">
         <v>411</v>
       </c>
-      <c r="B171" s="9" t="s">
+      <c r="B165" s="9" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A172" s="2"/>
-      <c r="B172" s="2"/>
-    </row>
+    <row r="166" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A166" s="2"/>
+      <c r="B166" s="2"/>
+    </row>
+    <row r="167" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A167" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B167" s="7">
+        <v>2000</v>
+      </c>
+      <c r="C167" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A168" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B168">
+        <v>1</v>
+      </c>
+      <c r="C168" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A169" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B169" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C169" s="6"/>
+    </row>
+    <row r="170" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A170" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B170" s="7">
+        <v>3</v>
+      </c>
+      <c r="C170" s="6"/>
+    </row>
+    <row r="171" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A171" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B171" s="7">
+        <v>3</v>
+      </c>
+      <c r="C171" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" ht="14.5"/>
     <row r="173" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A173" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B173" s="7">
-        <v>2000</v>
-      </c>
-      <c r="C173" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="174" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A174" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B174">
-        <v>1</v>
-      </c>
-      <c r="C174" t="s">
-        <v>61</v>
-      </c>
-    </row>
+      <c r="A173" t="s">
+        <v>91</v>
+      </c>
+      <c r="B173" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="175" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A175" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B175" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="C175" s="6"/>
+      <c r="A175" t="s">
+        <v>108</v>
+      </c>
+      <c r="B175" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="176" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A176" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B176" s="7">
-        <v>3</v>
-      </c>
-      <c r="C176" s="6"/>
-    </row>
-    <row r="177" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A177" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B177" s="7">
-        <v>3</v>
-      </c>
-      <c r="C177" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3" ht="14.5"/>
+      <c r="A176" t="s">
+        <v>96</v>
+      </c>
+      <c r="B176" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="178" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A178" t="s">
+        <v>110</v>
+      </c>
+      <c r="B178" t="s">
+        <v>113</v>
+      </c>
+    </row>
     <row r="179" spans="1:3" ht="14.25" customHeight="1">
       <c r="A179" t="s">
-        <v>91</v>
-      </c>
-      <c r="B179" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>116</v>
+      </c>
+      <c r="B179" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A180" t="s">
+        <v>111</v>
+      </c>
+      <c r="B180" t="s">
+        <v>112</v>
+      </c>
+    </row>
     <row r="181" spans="1:3" ht="14.25" customHeight="1">
       <c r="A181" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="B181" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="182" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A182" t="s">
-        <v>96</v>
-      </c>
-      <c r="B182" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="183" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="183" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A183" t="s">
+        <v>505</v>
+      </c>
+      <c r="B183">
+        <v>5</v>
+      </c>
+      <c r="C183" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="184" spans="1:3" ht="14.25" customHeight="1">
       <c r="A184" t="s">
-        <v>110</v>
-      </c>
-      <c r="B184" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="B184">
+        <v>2</v>
       </c>
     </row>
     <row r="185" spans="1:3" ht="14.25" customHeight="1">
       <c r="A185" t="s">
-        <v>116</v>
-      </c>
-      <c r="B185" t="s">
-        <v>118</v>
+        <v>115</v>
+      </c>
+      <c r="B185">
+        <v>40000</v>
+      </c>
+      <c r="C185" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="186" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A186" t="s">
-        <v>111</v>
-      </c>
-      <c r="B186" t="s">
-        <v>112</v>
-      </c>
+      <c r="A186" s="6"/>
+      <c r="B186" s="7"/>
     </row>
     <row r="187" spans="1:3" ht="14.25" customHeight="1">
       <c r="A187" t="s">
-        <v>117</v>
-      </c>
-      <c r="B187" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="188" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>105</v>
+      </c>
+      <c r="B187">
+        <v>30000</v>
+      </c>
+      <c r="C187" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A188" t="s">
+        <v>102</v>
+      </c>
+      <c r="B188">
+        <v>30000</v>
+      </c>
+      <c r="C188" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="189" spans="1:3" ht="14.25" customHeight="1">
       <c r="A189" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="B189">
-        <v>2</v>
+        <v>60000</v>
+      </c>
+      <c r="C189" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="190" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A190" t="s">
-        <v>115</v>
-      </c>
-      <c r="B190">
-        <v>40000</v>
-      </c>
-      <c r="C190" t="s">
+      <c r="A190" s="6"/>
+      <c r="B190" s="7"/>
+      <c r="C190" s="6"/>
+    </row>
+    <row r="191" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A191" t="s">
+        <v>74</v>
+      </c>
+      <c r="B191">
+        <v>2000</v>
+      </c>
+      <c r="C191" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="191" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A191" s="6"/>
-      <c r="B191" s="7"/>
     </row>
     <row r="192" spans="1:3" ht="14.25" customHeight="1">
       <c r="A192" t="s">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="B192">
-        <v>30000</v>
-      </c>
-      <c r="C192" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
     </row>
     <row r="193" spans="1:3" ht="14.25" customHeight="1">
       <c r="A193" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="B193">
-        <v>30000</v>
+        <v>1</v>
       </c>
       <c r="C193" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="195" spans="1:3" ht="15" customHeight="1">
+      <c r="A195" t="s">
+        <v>75</v>
+      </c>
+      <c r="B195">
+        <v>2000</v>
+      </c>
+      <c r="C195" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="194" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A194" t="s">
-        <v>106</v>
-      </c>
-      <c r="B194">
-        <v>60000</v>
-      </c>
-      <c r="C194" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="195" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A195" s="6"/>
-      <c r="B195" s="7"/>
-      <c r="C195" s="6"/>
     </row>
     <row r="196" spans="1:3" ht="14.25" customHeight="1">
       <c r="A196" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B196">
-        <v>2000</v>
-      </c>
-      <c r="C196" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" ht="17.5" customHeight="1">
+      <c r="A197" t="s">
+        <v>79</v>
+      </c>
+      <c r="B197">
+        <v>1</v>
+      </c>
+      <c r="C197" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" ht="17.5" customHeight="1"/>
+    <row r="199" spans="1:3" ht="17.5" customHeight="1">
+      <c r="A199" t="s">
+        <v>149</v>
+      </c>
+      <c r="B199">
+        <v>3000</v>
+      </c>
+      <c r="C199" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="197" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A197" t="s">
-        <v>76</v>
-      </c>
-      <c r="B197">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="198" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A198" t="s">
-        <v>77</v>
-      </c>
-      <c r="B198">
-        <v>1</v>
-      </c>
-      <c r="C198" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="199" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="200" spans="1:3" ht="15" customHeight="1">
-      <c r="A200" t="s">
-        <v>75</v>
-      </c>
-      <c r="B200">
-        <v>2000</v>
-      </c>
-      <c r="C200" t="s">
-        <v>72</v>
-      </c>
-    </row>
+    <row r="200" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="201" spans="1:3" ht="14.25" customHeight="1">
       <c r="A201" t="s">
-        <v>78</v>
-      </c>
-      <c r="B201">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="202" spans="1:3" ht="17.5" customHeight="1">
-      <c r="A202" t="s">
-        <v>79</v>
-      </c>
-      <c r="B202">
+        <v>120</v>
+      </c>
+      <c r="B201" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A202" s="6"/>
+      <c r="B202" s="7"/>
+      <c r="C202" s="6"/>
+    </row>
+    <row r="203" spans="1:3" ht="14" customHeight="1">
+      <c r="A203" t="s">
+        <v>121</v>
+      </c>
+      <c r="B203">
         <v>1</v>
       </c>
-      <c r="C202" t="s">
+      <c r="C203" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="203" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="204" spans="1:3" ht="17.5" customHeight="1">
-      <c r="A204" t="s">
-        <v>149</v>
-      </c>
-      <c r="B204">
-        <v>3000</v>
-      </c>
-      <c r="C204" t="s">
+    <row r="204" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="205" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A205" t="s">
+        <v>132</v>
+      </c>
+      <c r="B205">
+        <v>60000</v>
+      </c>
+      <c r="C205" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="205" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="206" spans="1:3" ht="14.25" customHeight="1">
       <c r="A206" t="s">
-        <v>120</v>
-      </c>
-      <c r="B206" t="s">
-        <v>410</v>
+        <v>131</v>
+      </c>
+      <c r="B206">
+        <v>60000</v>
+      </c>
+      <c r="C206" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="207" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A207" s="6"/>
-      <c r="B207" s="7"/>
-      <c r="C207" s="6"/>
-    </row>
-    <row r="208" spans="1:3" ht="14" customHeight="1">
+      <c r="A207" t="s">
+        <v>133</v>
+      </c>
+      <c r="B207">
+        <v>60000</v>
+      </c>
+      <c r="C207" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" ht="14.5" customHeight="1">
       <c r="A208" t="s">
-        <v>121</v>
+        <v>168</v>
       </c>
       <c r="B208">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C208" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="209" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="210" spans="1:3" ht="14.25" customHeight="1">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" ht="20.5" customHeight="1"/>
+    <row r="210" spans="1:3" ht="20.5" customHeight="1">
       <c r="A210" t="s">
-        <v>132</v>
+        <v>423</v>
       </c>
       <c r="B210">
-        <v>60000</v>
+        <v>5</v>
       </c>
       <c r="C210" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="211" spans="1:3" ht="14.25" customHeight="1">
+    <row r="211" spans="1:3" ht="14.5" customHeight="1">
       <c r="A211" t="s">
-        <v>131</v>
+        <v>424</v>
       </c>
       <c r="B211">
-        <v>60000</v>
+        <v>5</v>
       </c>
       <c r="C211" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="212" spans="1:3" ht="14.25" customHeight="1">
+    <row r="212" spans="1:3" ht="14.5" customHeight="1">
       <c r="A212" t="s">
-        <v>133</v>
+        <v>427</v>
       </c>
       <c r="B212">
-        <v>60000</v>
+        <v>5</v>
       </c>
       <c r="C212" t="s">
         <v>72</v>
@@ -3524,7 +3571,7 @@
     </row>
     <row r="213" spans="1:3" ht="14.5" customHeight="1">
       <c r="A213" t="s">
-        <v>168</v>
+        <v>444</v>
       </c>
       <c r="B213">
         <v>5</v>
@@ -3533,10 +3580,20 @@
         <v>72</v>
       </c>
     </row>
-    <row r="214" spans="1:3" ht="20.5" customHeight="1"/>
-    <row r="215" spans="1:3" ht="20.5" customHeight="1">
+    <row r="214" spans="1:3" ht="14.5" customHeight="1">
+      <c r="A214" t="s">
+        <v>453</v>
+      </c>
+      <c r="B214">
+        <v>5</v>
+      </c>
+      <c r="C214" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" ht="14.5" customHeight="1">
       <c r="A215" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="B215">
         <v>5</v>
@@ -3547,7 +3604,7 @@
     </row>
     <row r="216" spans="1:3" ht="14.5" customHeight="1">
       <c r="A216" t="s">
-        <v>424</v>
+        <v>463</v>
       </c>
       <c r="B216">
         <v>5</v>
@@ -3558,7 +3615,7 @@
     </row>
     <row r="217" spans="1:3" ht="14.5" customHeight="1">
       <c r="A217" t="s">
-        <v>427</v>
+        <v>466</v>
       </c>
       <c r="B217">
         <v>5</v>
@@ -3569,7 +3626,7 @@
     </row>
     <row r="218" spans="1:3" ht="14.5" customHeight="1">
       <c r="A218" t="s">
-        <v>444</v>
+        <v>467</v>
       </c>
       <c r="B218">
         <v>5</v>
@@ -3580,7 +3637,7 @@
     </row>
     <row r="219" spans="1:3" ht="14.5" customHeight="1">
       <c r="A219" t="s">
-        <v>453</v>
+        <v>468</v>
       </c>
       <c r="B219">
         <v>5</v>
@@ -3591,7 +3648,7 @@
     </row>
     <row r="220" spans="1:3" ht="14.5" customHeight="1">
       <c r="A220" t="s">
-        <v>460</v>
+        <v>473</v>
       </c>
       <c r="B220">
         <v>5</v>
@@ -3602,7 +3659,7 @@
     </row>
     <row r="221" spans="1:3" ht="14.5" customHeight="1">
       <c r="A221" t="s">
-        <v>463</v>
+        <v>474</v>
       </c>
       <c r="B221">
         <v>5</v>
@@ -3613,7 +3670,7 @@
     </row>
     <row r="222" spans="1:3" ht="14.5" customHeight="1">
       <c r="A222" t="s">
-        <v>466</v>
+        <v>481</v>
       </c>
       <c r="B222">
         <v>5</v>
@@ -3624,7 +3681,7 @@
     </row>
     <row r="223" spans="1:3" ht="14.5" customHeight="1">
       <c r="A223" t="s">
-        <v>467</v>
+        <v>482</v>
       </c>
       <c r="B223">
         <v>5</v>
@@ -3635,7 +3692,7 @@
     </row>
     <row r="224" spans="1:3" ht="14.5" customHeight="1">
       <c r="A224" t="s">
-        <v>468</v>
+        <v>485</v>
       </c>
       <c r="B224">
         <v>5</v>
@@ -3646,7 +3703,7 @@
     </row>
     <row r="225" spans="1:3" ht="14.5" customHeight="1">
       <c r="A225" t="s">
-        <v>473</v>
+        <v>490</v>
       </c>
       <c r="B225">
         <v>5</v>
@@ -3655,627 +3712,627 @@
         <v>72</v>
       </c>
     </row>
-    <row r="226" spans="1:3" ht="14.5" customHeight="1">
-      <c r="A226" t="s">
-        <v>474</v>
-      </c>
-      <c r="B226">
-        <v>5</v>
-      </c>
-      <c r="C226" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="227" spans="1:3" ht="14.5" customHeight="1">
+    <row r="226" spans="1:3" ht="14.5" customHeight="1"/>
+    <row r="227" spans="1:3" ht="15.5" customHeight="1">
       <c r="A227" t="s">
-        <v>481</v>
-      </c>
-      <c r="B227">
-        <v>5</v>
-      </c>
-      <c r="C227" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="228" spans="1:3" ht="14.5" customHeight="1">
+        <v>426</v>
+      </c>
+      <c r="B227" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" ht="13.5" customHeight="1">
       <c r="A228" t="s">
-        <v>482</v>
-      </c>
-      <c r="B228">
-        <v>5</v>
-      </c>
-      <c r="C228" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="229" spans="1:3" ht="14.5" customHeight="1">
+        <v>425</v>
+      </c>
+      <c r="B228" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" ht="16" customHeight="1">
       <c r="A229" t="s">
-        <v>485</v>
-      </c>
-      <c r="B229">
-        <v>5</v>
-      </c>
-      <c r="C229" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="230" spans="1:3" ht="14.5" customHeight="1">
+        <v>428</v>
+      </c>
+      <c r="B229" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" ht="16.5" customHeight="1">
       <c r="A230" t="s">
-        <v>490</v>
-      </c>
-      <c r="B230">
-        <v>5</v>
-      </c>
-      <c r="C230" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="231" spans="1:3" ht="14.5" customHeight="1"/>
-    <row r="232" spans="1:3" ht="15.5" customHeight="1">
+        <v>429</v>
+      </c>
+      <c r="B230" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A231" t="s">
+        <v>430</v>
+      </c>
+      <c r="B231" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" ht="13.5" customHeight="1">
       <c r="A232" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="B232" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="233" spans="1:3" ht="13.5" customHeight="1">
       <c r="A233" t="s">
-        <v>425</v>
+        <v>438</v>
       </c>
       <c r="B233" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="234" spans="1:3" ht="16" customHeight="1">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" ht="13.5" customHeight="1">
       <c r="A234" t="s">
-        <v>428</v>
+        <v>440</v>
       </c>
       <c r="B234" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="235" spans="1:3" ht="16.5" customHeight="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" ht="13.5" customHeight="1">
       <c r="A235" t="s">
-        <v>429</v>
+        <v>442</v>
       </c>
       <c r="B235" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
     </row>
     <row r="236" spans="1:3" ht="13.5" customHeight="1">
       <c r="A236" t="s">
-        <v>430</v>
+        <v>445</v>
       </c>
       <c r="B236" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="237" spans="1:3" ht="13.5" customHeight="1">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" ht="14.5" customHeight="1">
       <c r="A237" t="s">
-        <v>431</v>
+        <v>447</v>
       </c>
       <c r="B237" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="238" spans="1:3" ht="13.5" customHeight="1">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" ht="14.5" customHeight="1">
       <c r="A238" t="s">
-        <v>438</v>
+        <v>449</v>
       </c>
       <c r="B238" t="s">
-        <v>439</v>
+        <v>450</v>
       </c>
     </row>
     <row r="239" spans="1:3" ht="13.5" customHeight="1">
       <c r="A239" t="s">
-        <v>440</v>
+        <v>457</v>
       </c>
       <c r="B239" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="240" spans="1:3" ht="13.5" customHeight="1">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" ht="14.5" customHeight="1">
       <c r="A240" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="B240" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2" ht="13.5" customHeight="1">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" ht="15" customHeight="1">
       <c r="A241" t="s">
-        <v>445</v>
+        <v>459</v>
       </c>
       <c r="B241" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" ht="14.5" customHeight="1">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" ht="13.5" customHeight="1">
       <c r="A242" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="B242" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2" ht="14.5" customHeight="1">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" ht="13" customHeight="1">
       <c r="A243" t="s">
-        <v>449</v>
+        <v>461</v>
       </c>
       <c r="B243" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" ht="13.5" customHeight="1">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" ht="17" customHeight="1">
       <c r="A244" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="B244" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" ht="14.5" customHeight="1">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" ht="17" customHeight="1">
       <c r="A245" t="s">
-        <v>458</v>
+        <v>469</v>
       </c>
       <c r="B245" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" ht="15" customHeight="1">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" ht="17" customHeight="1">
       <c r="A246" t="s">
-        <v>459</v>
+        <v>471</v>
       </c>
       <c r="B246" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2" ht="13.5" customHeight="1">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" ht="17" customHeight="1">
       <c r="A247" t="s">
-        <v>455</v>
+        <v>475</v>
       </c>
       <c r="B247" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" ht="13" customHeight="1">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" ht="17" customHeight="1">
       <c r="A248" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="B248" t="s">
-        <v>462</v>
+        <v>478</v>
       </c>
     </row>
     <row r="249" spans="1:2" ht="17" customHeight="1">
       <c r="A249" t="s">
-        <v>464</v>
+        <v>479</v>
       </c>
       <c r="B249" t="s">
-        <v>465</v>
+        <v>480</v>
       </c>
     </row>
     <row r="250" spans="1:2" ht="17" customHeight="1">
       <c r="A250" t="s">
-        <v>469</v>
+        <v>483</v>
       </c>
       <c r="B250" t="s">
-        <v>470</v>
+        <v>484</v>
       </c>
     </row>
     <row r="251" spans="1:2" ht="17" customHeight="1">
       <c r="A251" t="s">
-        <v>471</v>
+        <v>486</v>
       </c>
       <c r="B251" t="s">
-        <v>472</v>
+        <v>487</v>
       </c>
     </row>
     <row r="252" spans="1:2" ht="17" customHeight="1">
       <c r="A252" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="B252" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="253" spans="1:2" ht="17" customHeight="1">
-      <c r="A253" t="s">
-        <v>477</v>
-      </c>
-      <c r="B253" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2" ht="17" customHeight="1">
-      <c r="A254" t="s">
-        <v>479</v>
-      </c>
-      <c r="B254" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" ht="17" customHeight="1">
-      <c r="A255" t="s">
-        <v>483</v>
-      </c>
-      <c r="B255" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2" ht="17" customHeight="1">
-      <c r="A256" t="s">
-        <v>486</v>
-      </c>
-      <c r="B256" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="257" spans="1:3" ht="17" customHeight="1">
-      <c r="A257" t="s">
-        <v>488</v>
+        <v>489</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" ht="17" customHeight="1"/>
+    <row r="254" spans="1:2" ht="17" customHeight="1"/>
+    <row r="255" spans="1:2" ht="17" customHeight="1"/>
+    <row r="256" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="257" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A257" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="B257" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="258" spans="1:3" ht="17" customHeight="1"/>
-    <row r="259" spans="1:3" ht="17" customHeight="1"/>
-    <row r="260" spans="1:3" ht="17" customHeight="1"/>
-    <row r="261" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="262" spans="1:3" ht="14.25" customHeight="1">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3" ht="17.5" customHeight="1"/>
+    <row r="259" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A259" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B259" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A260" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B260" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A261" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B261" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="A262" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B262" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="263" spans="1:3" ht="17.5" customHeight="1"/>
+        <v>56</v>
+      </c>
+      <c r="B262" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" s="6" customFormat="1" ht="14.5"/>
     <row r="264" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="A264" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B264" s="6" t="s">
-        <v>52</v>
+        <v>57</v>
+      </c>
+      <c r="B264" s="7" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="265" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="A265" s="6" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B265" s="7" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
     </row>
     <row r="266" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="A266" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B266" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="267" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A267" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B267" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="268" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="269" spans="1:3" s="6" customFormat="1" ht="14.5">
+        <v>60</v>
+      </c>
+      <c r="B266" s="7">
+        <v>60</v>
+      </c>
+      <c r="C266" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="268" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A268" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B268" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C268" s="6"/>
+    </row>
+    <row r="269" spans="1:3" ht="14.25" customHeight="1">
       <c r="A269" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B269" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="270" spans="1:3" s="6" customFormat="1" ht="14.5">
+        <v>59</v>
+      </c>
+      <c r="B269" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C269" s="6"/>
+    </row>
+    <row r="270" spans="1:3" ht="14.25" customHeight="1">
       <c r="A270" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B270" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="271" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A271" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B271" s="7">
+      <c r="B270" s="7">
         <v>60</v>
       </c>
-      <c r="C271" s="6" t="s">
+      <c r="C270" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="272" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="271" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A271" s="6"/>
+      <c r="B271" s="6"/>
+      <c r="C271" s="6"/>
+    </row>
+    <row r="272" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A272" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B272" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C272" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="273" spans="1:3" ht="14.25" customHeight="1">
       <c r="A273" s="6" t="s">
-        <v>57</v>
+        <v>135</v>
       </c>
       <c r="B273" s="7" t="s">
-        <v>58</v>
+        <v>335</v>
       </c>
       <c r="C273" s="6"/>
     </row>
     <row r="274" spans="1:3" ht="14.25" customHeight="1">
       <c r="A274" s="6" t="s">
-        <v>59</v>
+        <v>136</v>
       </c>
       <c r="B274" s="8" t="s">
-        <v>69</v>
+        <v>336</v>
       </c>
       <c r="C274" s="6"/>
     </row>
     <row r="275" spans="1:3" ht="14.25" customHeight="1">
       <c r="A275" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B275" s="7">
-        <v>60</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="B275" s="6"/>
       <c r="C275" s="6" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
     </row>
     <row r="276" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A276" s="6"/>
-      <c r="B276" s="6"/>
-      <c r="C276" s="6"/>
-    </row>
-    <row r="277" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A277" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="B277" s="5" t="s">
+      <c r="A276" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B276" s="7">
+        <v>60000</v>
+      </c>
+      <c r="C276" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="278" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A278" t="s">
+        <v>137</v>
+      </c>
+      <c r="B278" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="C277" s="6" t="s">
+      <c r="C278" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="278" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A278" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="B278" s="7" t="s">
-        <v>335</v>
-      </c>
-      <c r="C278" s="6"/>
-    </row>
     <row r="279" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A279" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="B279" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="C279" s="6"/>
+      <c r="A279" t="s">
+        <v>138</v>
+      </c>
+      <c r="B279" s="7" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="280" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A280" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B280" s="6"/>
-      <c r="C280" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="281" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A281" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B281" s="7">
-        <v>60000</v>
-      </c>
-      <c r="C281" s="6" t="s">
+      <c r="A280" t="s">
+        <v>139</v>
+      </c>
+      <c r="B280" s="8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" ht="14" customHeight="1"/>
+    <row r="282" spans="1:3" ht="14" customHeight="1"/>
+    <row r="283" spans="1:3" ht="14" customHeight="1"/>
+    <row r="284" spans="1:3" ht="14" customHeight="1">
+      <c r="A284" t="s">
+        <v>165</v>
+      </c>
+      <c r="B284" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3" ht="14" customHeight="1">
+      <c r="A285" t="s">
+        <v>169</v>
+      </c>
+      <c r="B285" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" ht="14" customHeight="1">
+      <c r="A286" t="s">
+        <v>171</v>
+      </c>
+      <c r="B286" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" ht="14" customHeight="1"/>
+    <row r="289" spans="1:3" ht="14" customHeight="1"/>
+    <row r="290" spans="1:3" ht="14" customHeight="1"/>
+    <row r="291" spans="1:3" ht="15" customHeight="1">
+      <c r="B291" s="12"/>
+    </row>
+    <row r="292" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="293" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="294" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="295" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="296" spans="1:3" ht="15" customHeight="1">
+      <c r="B296" s="12"/>
+    </row>
+    <row r="297" spans="1:3" ht="15" customHeight="1">
+      <c r="B297" s="12"/>
+    </row>
+    <row r="298" spans="1:3" ht="15" customHeight="1">
+      <c r="B298" s="12"/>
+    </row>
+    <row r="299" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B299" s="2"/>
+    </row>
+    <row r="300" spans="1:3" ht="15" customHeight="1">
+      <c r="B300" s="2"/>
+    </row>
+    <row r="301" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A301" t="s">
+        <v>180</v>
+      </c>
+      <c r="B301" s="2">
+        <v>5</v>
+      </c>
+      <c r="C301" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="282" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="283" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A283" t="s">
-        <v>137</v>
-      </c>
-      <c r="B283" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="C283" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="284" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A284" t="s">
-        <v>138</v>
-      </c>
-      <c r="B284" s="7" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="285" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A285" t="s">
-        <v>139</v>
-      </c>
-      <c r="B285" s="8" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="286" spans="1:3" ht="14" customHeight="1"/>
-    <row r="287" spans="1:3" ht="14" customHeight="1"/>
-    <row r="288" spans="1:3" ht="14" customHeight="1"/>
-    <row r="289" spans="1:2" ht="14" customHeight="1">
-      <c r="A289" t="s">
-        <v>165</v>
-      </c>
-      <c r="B289" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" ht="14" customHeight="1">
-      <c r="A290" t="s">
-        <v>169</v>
-      </c>
-      <c r="B290" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2" ht="14" customHeight="1">
-      <c r="A291" t="s">
-        <v>171</v>
-      </c>
-      <c r="B291" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="292" spans="1:2" ht="14" customHeight="1"/>
-    <row r="294" spans="1:2" ht="14" customHeight="1"/>
-    <row r="295" spans="1:2" ht="14" customHeight="1"/>
-    <row r="296" spans="1:2" ht="15" customHeight="1">
-      <c r="B296" s="12"/>
-    </row>
-    <row r="297" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="298" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="299" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="300" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="301" spans="1:2" ht="15" customHeight="1">
-      <c r="B301" s="12"/>
-    </row>
-    <row r="302" spans="1:2" ht="15" customHeight="1">
-      <c r="B302" s="12"/>
-    </row>
-    <row r="303" spans="1:2" ht="15" customHeight="1">
-      <c r="B303" s="12"/>
-    </row>
-    <row r="304" spans="1:2" ht="14.25" customHeight="1">
-      <c r="B304" s="2"/>
-    </row>
-    <row r="305" spans="1:3" ht="15" customHeight="1">
-      <c r="B305" s="2"/>
-    </row>
-    <row r="306" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A306" t="s">
-        <v>180</v>
-      </c>
-      <c r="B306" s="2">
+    <row r="302" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A302" t="s">
+        <v>181</v>
+      </c>
+      <c r="B302" s="2">
         <v>5</v>
       </c>
-      <c r="C306" t="s">
+      <c r="C302" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="307" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A307" t="s">
-        <v>181</v>
-      </c>
-      <c r="B307" s="2">
+    <row r="303" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A303" t="s">
+        <v>184</v>
+      </c>
+      <c r="B303" s="2">
         <v>5</v>
       </c>
-      <c r="C307" t="s">
+      <c r="C303" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="308" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A308" t="s">
-        <v>184</v>
-      </c>
-      <c r="B308" s="2">
-        <v>5</v>
-      </c>
-      <c r="C308" t="s">
-        <v>48</v>
-      </c>
-    </row>
+    <row r="304" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="305" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="307" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="308" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="309" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="310" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="312" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="313" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="314" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="315" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="316" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="317" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A317" t="s">
+    <row r="311" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="312" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A312" t="s">
         <v>401</v>
       </c>
-      <c r="B317" t="s">
+      <c r="B312" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="318" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A318" t="s">
+    <row r="313" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A313" t="s">
         <v>182</v>
       </c>
-      <c r="B318" t="s">
+      <c r="B313" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="319" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A319" t="s">
+    <row r="314" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A314" t="s">
         <v>183</v>
       </c>
-      <c r="B319" t="s">
+      <c r="B314" t="s">
         <v>187</v>
       </c>
     </row>
+    <row r="315" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A315" t="s">
+        <v>185</v>
+      </c>
+      <c r="B315" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A316" t="s">
+        <v>276</v>
+      </c>
+      <c r="B316" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="318" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="319" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="320" spans="1:3" ht="14.25" customHeight="1">
       <c r="A320" t="s">
-        <v>185</v>
-      </c>
-      <c r="B320" t="s">
-        <v>188</v>
+        <v>189</v>
+      </c>
+      <c r="B320">
+        <v>5</v>
+      </c>
+      <c r="C320" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="321" spans="1:3" ht="14.25" customHeight="1">
       <c r="A321" t="s">
-        <v>276</v>
+        <v>190</v>
       </c>
       <c r="B321" t="s">
-        <v>277</v>
+        <v>191</v>
       </c>
     </row>
     <row r="322" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="323" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="324" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="325" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A325" t="s">
-        <v>189</v>
-      </c>
-      <c r="B325">
+    <row r="324" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A324" t="s">
+        <v>192</v>
+      </c>
+      <c r="B324">
         <v>5</v>
       </c>
-      <c r="C325" t="s">
+      <c r="C324" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="326" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A326" t="s">
-        <v>190</v>
-      </c>
-      <c r="B326" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="327" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="328" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="325" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="326" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="327" spans="1:3" ht="14" customHeight="1">
+      <c r="A327" t="s">
+        <v>344</v>
+      </c>
+      <c r="B327">
+        <v>100</v>
+      </c>
+      <c r="C327" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A328" t="s">
+        <v>343</v>
+      </c>
+      <c r="B328">
+        <v>100</v>
+      </c>
+      <c r="C328" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="329" spans="1:3" ht="14.25" customHeight="1">
       <c r="A329" t="s">
-        <v>192</v>
+        <v>347</v>
       </c>
       <c r="B329">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="C329" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="330" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="331" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="332" spans="1:3" ht="14" customHeight="1">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="330" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A330" t="s">
+        <v>350</v>
+      </c>
+      <c r="B330">
+        <v>100</v>
+      </c>
+      <c r="C330" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="331" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A331" t="s">
+        <v>353</v>
+      </c>
+      <c r="B331">
+        <v>100</v>
+      </c>
+      <c r="C331" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="332" spans="1:3" ht="14.25" customHeight="1">
       <c r="A332" t="s">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="B332">
         <v>100</v>
@@ -4286,7 +4343,7 @@
     </row>
     <row r="333" spans="1:3" ht="14.25" customHeight="1">
       <c r="A333" t="s">
-        <v>343</v>
+        <v>359</v>
       </c>
       <c r="B333">
         <v>100</v>
@@ -4297,7 +4354,7 @@
     </row>
     <row r="334" spans="1:3" ht="14.25" customHeight="1">
       <c r="A334" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
       <c r="B334">
         <v>100</v>
@@ -4308,7 +4365,7 @@
     </row>
     <row r="335" spans="1:3" ht="14.25" customHeight="1">
       <c r="A335" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="B335">
         <v>100</v>
@@ -4317,154 +4374,124 @@
         <v>72</v>
       </c>
     </row>
-    <row r="336" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A336" t="s">
-        <v>353</v>
-      </c>
-      <c r="B336">
-        <v>100</v>
-      </c>
-      <c r="C336" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="337" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A337" t="s">
-        <v>356</v>
-      </c>
-      <c r="B337">
-        <v>100</v>
-      </c>
-      <c r="C337" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="338" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A338" t="s">
-        <v>359</v>
-      </c>
-      <c r="B338">
-        <v>100</v>
-      </c>
-      <c r="C338" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="339" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A339" t="s">
-        <v>362</v>
-      </c>
-      <c r="B339">
-        <v>100</v>
-      </c>
-      <c r="C339" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="340" spans="1:3" ht="14.25" customHeight="1">
+    <row r="336" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="337" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="338" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="339" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="340" spans="1:2" ht="14.25" customHeight="1">
       <c r="A340" t="s">
-        <v>365</v>
-      </c>
-      <c r="B340">
-        <v>100</v>
-      </c>
-      <c r="C340" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="341" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="342" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="343" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="344" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="345" spans="1:3" ht="14.25" customHeight="1">
+        <v>341</v>
+      </c>
+      <c r="B340" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A341" t="s">
+        <v>345</v>
+      </c>
+      <c r="B341" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="342" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A342" t="s">
+        <v>348</v>
+      </c>
+      <c r="B342" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A343" t="s">
+        <v>351</v>
+      </c>
+      <c r="B343" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A344" t="s">
+        <v>354</v>
+      </c>
+      <c r="B344" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="345" spans="1:2" ht="14.25" customHeight="1">
       <c r="A345" t="s">
-        <v>341</v>
+        <v>357</v>
       </c>
       <c r="B345" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="346" spans="1:3" ht="14.25" customHeight="1">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2" ht="14.25" customHeight="1">
       <c r="A346" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
       <c r="B346" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="347" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A347" t="s">
-        <v>348</v>
-      </c>
-      <c r="B347" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="348" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A348" t="s">
-        <v>351</v>
-      </c>
-      <c r="B348" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="349" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A349" t="s">
-        <v>354</v>
-      </c>
-      <c r="B349" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="350" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A350" t="s">
-        <v>357</v>
-      </c>
-      <c r="B350" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="351" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A351" t="s">
-        <v>360</v>
-      </c>
-      <c r="B351" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="352" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A352" s="6" t="s">
+    <row r="347" spans="1:2" s="6" customFormat="1" ht="14.5">
+      <c r="A347" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="B352" s="6" t="s">
+      <c r="B347" s="6" t="s">
         <v>364</v>
       </c>
     </row>
+    <row r="348" spans="1:2" s="6" customFormat="1" ht="14.5">
+      <c r="A348" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="B348" s="7" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2" s="6" customFormat="1" ht="14.5">
+      <c r="B349" s="7"/>
+    </row>
+    <row r="350" spans="1:2" s="6" customFormat="1" ht="14.5">
+      <c r="B350" s="7"/>
+    </row>
+    <row r="351" spans="1:2" s="6" customFormat="1" ht="14.5"/>
+    <row r="352" spans="1:2" s="6" customFormat="1" ht="14.5">
+      <c r="B352" s="7"/>
+    </row>
     <row r="353" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A353" s="6" t="s">
-        <v>366</v>
-      </c>
-      <c r="B353" s="7" t="s">
-        <v>367</v>
-      </c>
+      <c r="B353" s="7"/>
     </row>
     <row r="354" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="B354" s="7"/>
     </row>
-    <row r="355" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B355" s="7"/>
-    </row>
-    <row r="356" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="357" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B357" s="7"/>
-    </row>
-    <row r="358" spans="1:3" s="6" customFormat="1" ht="14.5">
+    <row r="355" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="356" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A356" s="6"/>
+      <c r="B356" s="7"/>
+      <c r="C356" s="6"/>
+    </row>
+    <row r="357" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A357" s="6"/>
+      <c r="B357" s="8"/>
+      <c r="C357" s="6"/>
+    </row>
+    <row r="358" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A358" s="6"/>
       <c r="B358" s="7"/>
-    </row>
-    <row r="359" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B359" s="7"/>
-    </row>
-    <row r="360" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="C358" s="6"/>
+    </row>
+    <row r="359" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A359" s="6"/>
+      <c r="B359" s="6"/>
+      <c r="C359" s="6"/>
+    </row>
+    <row r="360" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A360" s="6"/>
+      <c r="B360" s="5"/>
+      <c r="C360" s="6"/>
+    </row>
     <row r="361" spans="1:3" ht="14.25" customHeight="1">
       <c r="A361" s="6"/>
       <c r="B361" s="7"/>
@@ -4477,62 +4504,42 @@
     </row>
     <row r="363" spans="1:3" ht="14.25" customHeight="1">
       <c r="A363" s="6"/>
-      <c r="B363" s="7"/>
+      <c r="B363" s="6"/>
       <c r="C363" s="6"/>
     </row>
     <row r="364" spans="1:3" ht="14.25" customHeight="1">
       <c r="A364" s="6"/>
-      <c r="B364" s="6"/>
+      <c r="B364" s="7"/>
       <c r="C364" s="6"/>
     </row>
-    <row r="365" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A365" s="6"/>
-      <c r="B365" s="5"/>
-      <c r="C365" s="6"/>
-    </row>
+    <row r="365" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="366" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A366" s="6"/>
-      <c r="B366" s="7"/>
-      <c r="C366" s="6"/>
+      <c r="B366" s="5"/>
     </row>
     <row r="367" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A367" s="6"/>
-      <c r="B367" s="8"/>
-      <c r="C367" s="6"/>
+      <c r="B367" s="7"/>
     </row>
     <row r="368" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A368" s="6"/>
-      <c r="B368" s="6"/>
-      <c r="C368" s="6"/>
-    </row>
-    <row r="369" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A369" s="6"/>
-      <c r="B369" s="7"/>
-      <c r="C369" s="6"/>
-    </row>
-    <row r="370" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="371" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B371" s="5"/>
-    </row>
-    <row r="372" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B372" s="7"/>
-    </row>
-    <row r="373" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B373" s="8"/>
-    </row>
-    <row r="374" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="375" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A375" s="6"/>
-    </row>
-    <row r="376" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="377" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="378" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="379" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="380" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="381" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="382" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="383" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="384" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="B368" s="8"/>
+    </row>
+    <row r="369" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="370" spans="1:1" ht="14.25" customHeight="1">
+      <c r="A370" s="6"/>
+    </row>
+    <row r="371" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="372" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="373" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="374" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="375" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="376" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="377" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="378" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="379" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="380" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="381" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="382" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="383" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="384" spans="1:1" ht="14.25" customHeight="1"/>
     <row r="385" ht="14.25" customHeight="1"/>
     <row r="386" ht="14.25" customHeight="1"/>
     <row r="387" ht="14.25" customHeight="1"/>
@@ -5375,11 +5382,6 @@
     <row r="1224" ht="14.25" customHeight="1"/>
     <row r="1225" ht="14.25" customHeight="1"/>
     <row r="1226" ht="14.25" customHeight="1"/>
-    <row r="1227" ht="14.25" customHeight="1"/>
-    <row r="1228" ht="14.25" customHeight="1"/>
-    <row r="1229" ht="14.25" customHeight="1"/>
-    <row r="1230" ht="14.25" customHeight="1"/>
-    <row r="1231" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Entry Transaction Fields Workflow
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harih\OneDrive\Documents\UiPath\Invoices\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1726B9EA-7336-46E7-8547-53C7D6943CAC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C736D1-22DD-48CE-8A45-0920372337F5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="508">
   <si>
     <t>Name</t>
   </si>
@@ -518,9 +518,6 @@
     <t>SE_ErrMsg_MaxRetry</t>
   </si>
   <si>
-    <t>Treasury Confirmation - Error Occurred</t>
-  </si>
-  <si>
     <t>Status_InProgress</t>
   </si>
   <si>
@@ -1542,6 +1539,15 @@
   </si>
   <si>
     <t>TimeOut_IEModeEdgeBrowser</t>
+  </si>
+  <si>
+    <t>RetryNum_GLAccountError_F4Key</t>
+  </si>
+  <si>
+    <t>RetryInterval_GLAccountError_F4Key</t>
+  </si>
+  <si>
+    <t>Invoice Transactions - Error Occurred</t>
   </si>
 </sst>
 </file>
@@ -1594,7 +1600,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1617,7 +1623,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
@@ -1934,7 +1939,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1226"/>
+  <dimension ref="A1:Z1203"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="49.54296875" customWidth="1"/>
@@ -1987,7 +1992,7 @@
         <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -2049,10 +2054,10 @@
     </row>
     <row r="12" spans="1:26" ht="14.5">
       <c r="A12" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="15" customHeight="1">
@@ -2083,279 +2088,279 @@
     </row>
     <row r="16" spans="1:26" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>332</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>194</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.5">
       <c r="A24" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.5">
       <c r="A25" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.5">
       <c r="A26" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.5">
       <c r="A27" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.5">
       <c r="A28" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.5">
       <c r="A29" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.5">
       <c r="A30" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.5">
       <c r="A31" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.5">
       <c r="A32" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.5">
       <c r="A33" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.5">
       <c r="A34" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.5">
       <c r="A35" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.5">
       <c r="A36" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.5">
       <c r="A37" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.5">
       <c r="A38" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.5">
       <c r="A39" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.5">
       <c r="A40" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.5">
       <c r="A41" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.5">
       <c r="A42" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.5">
       <c r="A43" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.5">
       <c r="A44" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.5">
       <c r="A45" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.5">
       <c r="A46" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.5">
       <c r="A47" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.5">
       <c r="A48" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.5">
       <c r="A49" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.5">
       <c r="A50" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>3</v>
@@ -2363,135 +2368,135 @@
     </row>
     <row r="51" spans="1:2" ht="14.5">
       <c r="A51" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.5">
       <c r="A52" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.5">
       <c r="A53" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.5">
       <c r="A54" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.5">
       <c r="A55" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="14.5">
       <c r="A56" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.5">
       <c r="A57" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="14.5">
       <c r="A58" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.5">
       <c r="A59" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B59" s="2" t="s">
         <v>280</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="14.5">
       <c r="A60" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="14.5">
       <c r="A61" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B61" s="2" t="s">
         <v>284</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="14.5">
       <c r="A62" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>286</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="14.5">
       <c r="A63" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>288</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="14.5">
       <c r="A64" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B64" s="2" t="s">
         <v>290</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="14.5">
       <c r="A65" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B65" s="2" t="s">
         <v>292</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="14.5">
       <c r="A66" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>294</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="14.5">
       <c r="A67" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>3</v>
@@ -2499,290 +2504,290 @@
     </row>
     <row r="68" spans="1:2" ht="14.5">
       <c r="A68" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="14.5">
       <c r="A69" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="14.5">
       <c r="A70" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="14.5">
       <c r="A71" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="14.5">
       <c r="A72" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="14.5">
       <c r="A73" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="14.5">
       <c r="A74" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="B74" s="13" t="s">
-        <v>298</v>
+        <v>313</v>
+      </c>
+      <c r="B74" s="12" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="14.5">
       <c r="A75" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="B75" s="13" t="s">
-        <v>299</v>
+        <v>314</v>
+      </c>
+      <c r="B75" s="12" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="14.5">
       <c r="A76" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="B76" s="13" t="s">
-        <v>300</v>
+        <v>315</v>
+      </c>
+      <c r="B76" s="12" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="14.5">
       <c r="A77" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="B77" s="13" t="s">
-        <v>301</v>
+        <v>316</v>
+      </c>
+      <c r="B77" s="12" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="14.5">
       <c r="A78" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="B78" s="13" t="s">
-        <v>302</v>
+        <v>317</v>
+      </c>
+      <c r="B78" s="12" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="14.5">
       <c r="A79" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="B79" s="13" t="s">
-        <v>303</v>
+        <v>318</v>
+      </c>
+      <c r="B79" s="12" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="14.5">
       <c r="A80" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="B80" s="13" t="s">
-        <v>304</v>
+        <v>319</v>
+      </c>
+      <c r="B80" s="12" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="14.5">
       <c r="A81" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="B81" s="13" t="s">
-        <v>305</v>
+        <v>320</v>
+      </c>
+      <c r="B81" s="12" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="14.5">
       <c r="A82" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="B82" s="13" t="s">
-        <v>306</v>
+        <v>321</v>
+      </c>
+      <c r="B82" s="12" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="14.5">
       <c r="A83" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="B83" s="13" t="s">
-        <v>307</v>
+        <v>322</v>
+      </c>
+      <c r="B83" s="12" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="14.5">
       <c r="A84" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="B84" s="13" t="s">
-        <v>308</v>
+        <v>323</v>
+      </c>
+      <c r="B84" s="12" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="14.5">
       <c r="A85" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="B85" s="13" t="s">
-        <v>309</v>
+        <v>324</v>
+      </c>
+      <c r="B85" s="12" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="14.5">
       <c r="A86" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="B86" s="13" t="s">
-        <v>310</v>
+        <v>327</v>
+      </c>
+      <c r="B86" s="12" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="14.5">
       <c r="A87" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="B87" s="13" t="s">
-        <v>311</v>
+        <v>325</v>
+      </c>
+      <c r="B87" s="12" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="14.5">
       <c r="A88" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="B88" s="13" t="s">
-        <v>312</v>
+        <v>326</v>
+      </c>
+      <c r="B88" s="12" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="14.5">
       <c r="A89" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="B89" s="13" t="s">
-        <v>313</v>
+        <v>328</v>
+      </c>
+      <c r="B89" s="12" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="15" customHeight="1">
       <c r="A90" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B90" s="6" t="s">
         <v>368</v>
-      </c>
-      <c r="B90" s="6" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="14.5">
       <c r="A91" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="14.5">
       <c r="A92" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="14.5">
       <c r="A93" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="14.5">
       <c r="A94" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="14.5">
       <c r="A95" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="14.5">
       <c r="A96" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="14.5">
       <c r="A97" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="14.5">
       <c r="A98" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="14.5">
       <c r="A99" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="14.5">
       <c r="A100" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="14.5">
       <c r="A101" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="14.5">
       <c r="A102" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="14.5">
       <c r="A103" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="14.5">
@@ -2791,18 +2796,18 @@
     </row>
     <row r="106" spans="1:2" ht="14.5">
       <c r="A106" t="s">
+        <v>336</v>
+      </c>
+      <c r="B106" t="s">
         <v>337</v>
-      </c>
-      <c r="B106" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="15" customHeight="1">
       <c r="A107" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B107" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="14.5">
@@ -2860,7 +2865,7 @@
         <v>49</v>
       </c>
       <c r="B116" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="14.25" customHeight="1">
@@ -2868,13 +2873,13 @@
         <v>66</v>
       </c>
       <c r="B117" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="119" spans="1:2" ht="14.25" customHeight="1">
       <c r="A119" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="15" customHeight="1">
@@ -2927,50 +2932,50 @@
     </row>
     <row r="130" spans="1:2" ht="14.5">
       <c r="A130" t="s">
+        <v>394</v>
+      </c>
+      <c r="B130" t="s">
         <v>395</v>
-      </c>
-      <c r="B130" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="14.5">
       <c r="A131" t="s">
+        <v>398</v>
+      </c>
+      <c r="B131" t="s">
         <v>399</v>
-      </c>
-      <c r="B131" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="14.5">
       <c r="A132" t="s">
+        <v>396</v>
+      </c>
+      <c r="B132" t="s">
         <v>397</v>
-      </c>
-      <c r="B132" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="14.5">
       <c r="A133" t="s">
+        <v>402</v>
+      </c>
+      <c r="B133" t="s">
         <v>403</v>
-      </c>
-      <c r="B133" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="14.5">
       <c r="A134" t="s">
+        <v>404</v>
+      </c>
+      <c r="B134" t="s">
         <v>405</v>
-      </c>
-      <c r="B134" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="14.5">
       <c r="A135" t="s">
+        <v>406</v>
+      </c>
+      <c r="B135" t="s">
         <v>407</v>
-      </c>
-      <c r="B135" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="14.5">
@@ -2991,7 +2996,7 @@
     </row>
     <row r="138" spans="1:2" ht="14.5">
       <c r="A138" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B138" t="s">
         <v>93</v>
@@ -3007,18 +3012,18 @@
     </row>
     <row r="140" spans="1:2" s="9" customFormat="1" ht="14.5">
       <c r="A140" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B140" s="9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="141" spans="1:2" s="9" customFormat="1" ht="14.5">
       <c r="A141" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B141" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="142" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
@@ -3034,103 +3039,103 @@
         <v>123</v>
       </c>
       <c r="B143" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="14.25" customHeight="1">
       <c r="A144" t="s">
+        <v>412</v>
+      </c>
+      <c r="B144" s="9" t="s">
         <v>413</v>
-      </c>
-      <c r="B144" s="9" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="14.25" customHeight="1">
       <c r="A145" t="s">
+        <v>414</v>
+      </c>
+      <c r="B145" s="9" t="s">
         <v>415</v>
-      </c>
-      <c r="B145" s="9" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="14.5">
       <c r="A146" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B146" s="9" t="s">
         <v>417</v>
-      </c>
-      <c r="B146" s="9" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="14.5">
       <c r="A147" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B147" s="9" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="14.5">
       <c r="A148" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B148" s="9" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="14.5">
       <c r="A149" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="B149" s="9" t="s">
         <v>491</v>
-      </c>
-      <c r="B149" s="9" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="14.5">
       <c r="A150" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="B150" s="9" t="s">
         <v>493</v>
-      </c>
-      <c r="B150" s="9" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="14.5">
       <c r="A151" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="B151" s="9" t="s">
         <v>495</v>
-      </c>
-      <c r="B151" s="9" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="14.5">
       <c r="A152" s="2" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B152" s="9" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="153" spans="1:2" ht="14.5">
       <c r="A153" s="2" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B153" s="9" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="14.5">
       <c r="A154" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="B154" s="9" t="s">
         <v>501</v>
-      </c>
-      <c r="B154" s="9" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="14.5">
       <c r="A155" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="B155" s="9" t="s">
         <v>503</v>
-      </c>
-      <c r="B155" s="9" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="14.5">
@@ -3182,27 +3187,27 @@
       </c>
     </row>
     <row r="163" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A163" s="14" t="s">
+      <c r="A163" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="B163" s="14" t="s">
+      <c r="B163" s="13" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="164" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
       <c r="A164" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B164" s="9" t="s">
         <v>178</v>
-      </c>
-      <c r="B164" s="9" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="165" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
       <c r="A165" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="B165" s="9" t="s">
         <v>411</v>
-      </c>
-      <c r="B165" s="9" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="166" spans="1:3" ht="14.25" customHeight="1">
@@ -3322,7 +3327,7 @@
     <row r="182" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="183" spans="1:3" ht="14.25" customHeight="1">
       <c r="A183" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B183">
         <v>5</v>
@@ -3471,7 +3476,7 @@
         <v>120</v>
       </c>
       <c r="B201" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="202" spans="1:3" ht="14.25" customHeight="1">
@@ -3526,7 +3531,7 @@
     </row>
     <row r="208" spans="1:3" ht="14.5" customHeight="1">
       <c r="A208" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B208">
         <v>5</v>
@@ -3538,7 +3543,7 @@
     <row r="209" spans="1:3" ht="20.5" customHeight="1"/>
     <row r="210" spans="1:3" ht="20.5" customHeight="1">
       <c r="A210" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B210">
         <v>5</v>
@@ -3549,7 +3554,7 @@
     </row>
     <row r="211" spans="1:3" ht="14.5" customHeight="1">
       <c r="A211" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B211">
         <v>5</v>
@@ -3560,7 +3565,7 @@
     </row>
     <row r="212" spans="1:3" ht="14.5" customHeight="1">
       <c r="A212" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B212">
         <v>5</v>
@@ -3571,7 +3576,7 @@
     </row>
     <row r="213" spans="1:3" ht="14.5" customHeight="1">
       <c r="A213" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B213">
         <v>5</v>
@@ -3582,7 +3587,7 @@
     </row>
     <row r="214" spans="1:3" ht="14.5" customHeight="1">
       <c r="A214" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B214">
         <v>5</v>
@@ -3593,7 +3598,7 @@
     </row>
     <row r="215" spans="1:3" ht="14.5" customHeight="1">
       <c r="A215" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B215">
         <v>5</v>
@@ -3604,7 +3609,7 @@
     </row>
     <row r="216" spans="1:3" ht="14.5" customHeight="1">
       <c r="A216" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B216">
         <v>5</v>
@@ -3615,7 +3620,7 @@
     </row>
     <row r="217" spans="1:3" ht="14.5" customHeight="1">
       <c r="A217" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B217">
         <v>5</v>
@@ -3626,7 +3631,7 @@
     </row>
     <row r="218" spans="1:3" ht="14.5" customHeight="1">
       <c r="A218" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B218">
         <v>5</v>
@@ -3637,7 +3642,7 @@
     </row>
     <row r="219" spans="1:3" ht="14.5" customHeight="1">
       <c r="A219" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B219">
         <v>5</v>
@@ -3648,7 +3653,7 @@
     </row>
     <row r="220" spans="1:3" ht="14.5" customHeight="1">
       <c r="A220" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B220">
         <v>5</v>
@@ -3659,7 +3664,7 @@
     </row>
     <row r="221" spans="1:3" ht="14.5" customHeight="1">
       <c r="A221" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B221">
         <v>5</v>
@@ -3670,7 +3675,7 @@
     </row>
     <row r="222" spans="1:3" ht="14.5" customHeight="1">
       <c r="A222" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B222">
         <v>5</v>
@@ -3681,7 +3686,7 @@
     </row>
     <row r="223" spans="1:3" ht="14.5" customHeight="1">
       <c r="A223" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B223">
         <v>5</v>
@@ -3692,7 +3697,7 @@
     </row>
     <row r="224" spans="1:3" ht="14.5" customHeight="1">
       <c r="A224" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B224">
         <v>5</v>
@@ -3703,7 +3708,7 @@
     </row>
     <row r="225" spans="1:3" ht="14.5" customHeight="1">
       <c r="A225" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B225">
         <v>5</v>
@@ -3715,210 +3720,210 @@
     <row r="226" spans="1:3" ht="14.5" customHeight="1"/>
     <row r="227" spans="1:3" ht="15.5" customHeight="1">
       <c r="A227" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B227" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="228" spans="1:3" ht="13.5" customHeight="1">
       <c r="A228" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B228" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="229" spans="1:3" ht="16" customHeight="1">
       <c r="A229" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B229" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="230" spans="1:3" ht="16.5" customHeight="1">
       <c r="A230" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B230" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="231" spans="1:3" ht="13.5" customHeight="1">
       <c r="A231" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B231" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="232" spans="1:3" ht="13.5" customHeight="1">
       <c r="A232" t="s">
+        <v>430</v>
+      </c>
+      <c r="B232" t="s">
         <v>431</v>
-      </c>
-      <c r="B232" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="233" spans="1:3" ht="13.5" customHeight="1">
       <c r="A233" t="s">
+        <v>437</v>
+      </c>
+      <c r="B233" t="s">
         <v>438</v>
-      </c>
-      <c r="B233" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="234" spans="1:3" ht="13.5" customHeight="1">
       <c r="A234" t="s">
+        <v>439</v>
+      </c>
+      <c r="B234" t="s">
         <v>440</v>
-      </c>
-      <c r="B234" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="235" spans="1:3" ht="13.5" customHeight="1">
       <c r="A235" t="s">
+        <v>441</v>
+      </c>
+      <c r="B235" t="s">
         <v>442</v>
-      </c>
-      <c r="B235" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="236" spans="1:3" ht="13.5" customHeight="1">
       <c r="A236" t="s">
+        <v>444</v>
+      </c>
+      <c r="B236" t="s">
         <v>445</v>
-      </c>
-      <c r="B236" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="237" spans="1:3" ht="14.5" customHeight="1">
       <c r="A237" t="s">
+        <v>446</v>
+      </c>
+      <c r="B237" t="s">
         <v>447</v>
-      </c>
-      <c r="B237" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="238" spans="1:3" ht="14.5" customHeight="1">
       <c r="A238" t="s">
+        <v>448</v>
+      </c>
+      <c r="B238" t="s">
         <v>449</v>
-      </c>
-      <c r="B238" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="239" spans="1:3" ht="13.5" customHeight="1">
       <c r="A239" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B239" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="240" spans="1:3" ht="14.5" customHeight="1">
       <c r="A240" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B240" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="241" spans="1:2" ht="15" customHeight="1">
       <c r="A241" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B241" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="242" spans="1:2" ht="13.5" customHeight="1">
       <c r="A242" t="s">
+        <v>454</v>
+      </c>
+      <c r="B242" t="s">
         <v>455</v>
-      </c>
-      <c r="B242" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="243" spans="1:2" ht="13" customHeight="1">
       <c r="A243" t="s">
+        <v>460</v>
+      </c>
+      <c r="B243" t="s">
         <v>461</v>
-      </c>
-      <c r="B243" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="244" spans="1:2" ht="17" customHeight="1">
       <c r="A244" t="s">
+        <v>463</v>
+      </c>
+      <c r="B244" t="s">
         <v>464</v>
-      </c>
-      <c r="B244" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="245" spans="1:2" ht="17" customHeight="1">
       <c r="A245" t="s">
+        <v>468</v>
+      </c>
+      <c r="B245" t="s">
         <v>469</v>
-      </c>
-      <c r="B245" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="246" spans="1:2" ht="17" customHeight="1">
       <c r="A246" t="s">
+        <v>470</v>
+      </c>
+      <c r="B246" t="s">
         <v>471</v>
-      </c>
-      <c r="B246" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="247" spans="1:2" ht="17" customHeight="1">
       <c r="A247" t="s">
+        <v>474</v>
+      </c>
+      <c r="B247" t="s">
         <v>475</v>
-      </c>
-      <c r="B247" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="248" spans="1:2" ht="17" customHeight="1">
       <c r="A248" t="s">
+        <v>476</v>
+      </c>
+      <c r="B248" t="s">
         <v>477</v>
-      </c>
-      <c r="B248" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="249" spans="1:2" ht="17" customHeight="1">
       <c r="A249" t="s">
+        <v>478</v>
+      </c>
+      <c r="B249" t="s">
         <v>479</v>
-      </c>
-      <c r="B249" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="250" spans="1:2" ht="17" customHeight="1">
       <c r="A250" t="s">
+        <v>482</v>
+      </c>
+      <c r="B250" t="s">
         <v>483</v>
-      </c>
-      <c r="B250" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="251" spans="1:2" ht="17" customHeight="1">
       <c r="A251" t="s">
+        <v>485</v>
+      </c>
+      <c r="B251" t="s">
         <v>486</v>
-      </c>
-      <c r="B251" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="252" spans="1:2" ht="17" customHeight="1">
       <c r="A252" t="s">
+        <v>487</v>
+      </c>
+      <c r="B252" t="s">
         <v>488</v>
-      </c>
-      <c r="B252" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="253" spans="1:2" ht="17" customHeight="1"/>
@@ -4034,7 +4039,7 @@
         <v>134</v>
       </c>
       <c r="B272" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C272" s="6" t="s">
         <v>45</v>
@@ -4045,7 +4050,7 @@
         <v>135</v>
       </c>
       <c r="B273" s="7" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C273" s="6"/>
     </row>
@@ -4054,7 +4059,7 @@
         <v>136</v>
       </c>
       <c r="B274" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C274" s="6"/>
     </row>
@@ -4084,7 +4089,7 @@
         <v>137</v>
       </c>
       <c r="B278" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C278" s="6" t="s">
         <v>45</v>
@@ -4095,7 +4100,7 @@
         <v>138</v>
       </c>
       <c r="B279" s="7" t="s">
-        <v>164</v>
+        <v>507</v>
       </c>
     </row>
     <row r="280" spans="1:3" ht="14.25" customHeight="1">
@@ -4108,438 +4113,447 @@
     </row>
     <row r="281" spans="1:3" ht="14" customHeight="1"/>
     <row r="282" spans="1:3" ht="14" customHeight="1"/>
-    <row r="283" spans="1:3" ht="14" customHeight="1"/>
+    <row r="283" spans="1:3" ht="14" customHeight="1">
+      <c r="A283" t="s">
+        <v>164</v>
+      </c>
+      <c r="B283" t="s">
+        <v>165</v>
+      </c>
+    </row>
     <row r="284" spans="1:3" ht="14" customHeight="1">
       <c r="A284" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B284" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="285" spans="1:3" ht="14" customHeight="1">
       <c r="A285" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B285" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="286" spans="1:3" ht="14" customHeight="1">
-      <c r="A286" t="s">
         <v>171</v>
       </c>
-      <c r="B286" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="287" spans="1:3" ht="14" customHeight="1"/>
+    </row>
+    <row r="286" spans="1:3" ht="14" customHeight="1"/>
+    <row r="287" spans="1:3" ht="15" customHeight="1">
+      <c r="A287" t="s">
+        <v>505</v>
+      </c>
+      <c r="B287">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" ht="14" customHeight="1">
+      <c r="A288" t="s">
+        <v>506</v>
+      </c>
+      <c r="B288">
+        <v>1</v>
+      </c>
+      <c r="C288" t="s">
+        <v>61</v>
+      </c>
+    </row>
     <row r="289" spans="1:3" ht="14" customHeight="1"/>
-    <row r="290" spans="1:3" ht="14" customHeight="1"/>
-    <row r="291" spans="1:3" ht="15" customHeight="1">
-      <c r="B291" s="12"/>
-    </row>
-    <row r="292" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="293" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="290" spans="1:3" ht="15" customHeight="1">
+      <c r="B290" s="2"/>
+    </row>
+    <row r="291" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A291" t="s">
+        <v>179</v>
+      </c>
+      <c r="B291" s="2">
+        <v>5</v>
+      </c>
+      <c r="C291" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A292" t="s">
+        <v>180</v>
+      </c>
+      <c r="B292" s="2">
+        <v>5</v>
+      </c>
+      <c r="C292" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="293" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A293" t="s">
+        <v>183</v>
+      </c>
+      <c r="B293" s="2">
+        <v>5</v>
+      </c>
+      <c r="C293" t="s">
+        <v>48</v>
+      </c>
+    </row>
     <row r="294" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="295" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="296" spans="1:3" ht="15" customHeight="1">
-      <c r="B296" s="12"/>
-    </row>
-    <row r="297" spans="1:3" ht="15" customHeight="1">
-      <c r="B297" s="12"/>
-    </row>
-    <row r="298" spans="1:3" ht="15" customHeight="1">
-      <c r="B298" s="12"/>
+    <row r="296" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A296" t="s">
+        <v>400</v>
+      </c>
+      <c r="B296" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A297" t="s">
+        <v>181</v>
+      </c>
+      <c r="B297" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A298" t="s">
+        <v>182</v>
+      </c>
+      <c r="B298" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="299" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B299" s="2"/>
-    </row>
-    <row r="300" spans="1:3" ht="15" customHeight="1">
-      <c r="B300" s="2"/>
-    </row>
-    <row r="301" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A301" t="s">
-        <v>180</v>
-      </c>
-      <c r="B301" s="2">
-        <v>5</v>
-      </c>
-      <c r="C301" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="302" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A302" t="s">
-        <v>181</v>
-      </c>
-      <c r="B302" s="2">
-        <v>5</v>
-      </c>
-      <c r="C302" t="s">
-        <v>48</v>
-      </c>
-    </row>
+      <c r="A299" t="s">
+        <v>184</v>
+      </c>
+      <c r="B299" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A300" t="s">
+        <v>275</v>
+      </c>
+      <c r="B300" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="302" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="303" spans="1:3" ht="14.25" customHeight="1">
       <c r="A303" t="s">
-        <v>184</v>
-      </c>
-      <c r="B303" s="2">
+        <v>188</v>
+      </c>
+      <c r="B303">
         <v>5</v>
       </c>
       <c r="C303" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="304" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="304" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A304" t="s">
+        <v>189</v>
+      </c>
+      <c r="B304" t="s">
+        <v>190</v>
+      </c>
+    </row>
     <row r="305" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="307" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="308" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="309" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="310" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="311" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="306" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A306" t="s">
+        <v>191</v>
+      </c>
+      <c r="B306">
+        <v>5</v>
+      </c>
+      <c r="C306" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" ht="14" customHeight="1">
+      <c r="A307" t="s">
+        <v>343</v>
+      </c>
+      <c r="B307">
+        <v>100</v>
+      </c>
+      <c r="C307" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A308" t="s">
+        <v>342</v>
+      </c>
+      <c r="B308">
+        <v>100</v>
+      </c>
+      <c r="C308" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A309" t="s">
+        <v>346</v>
+      </c>
+      <c r="B309">
+        <v>100</v>
+      </c>
+      <c r="C309" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A310" t="s">
+        <v>349</v>
+      </c>
+      <c r="B310">
+        <v>100</v>
+      </c>
+      <c r="C310" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A311" t="s">
+        <v>352</v>
+      </c>
+      <c r="B311">
+        <v>100</v>
+      </c>
+      <c r="C311" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="312" spans="1:3" ht="14.25" customHeight="1">
       <c r="A312" t="s">
-        <v>401</v>
-      </c>
-      <c r="B312" t="s">
-        <v>402</v>
+        <v>355</v>
+      </c>
+      <c r="B312">
+        <v>100</v>
+      </c>
+      <c r="C312" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="313" spans="1:3" ht="14.25" customHeight="1">
       <c r="A313" t="s">
-        <v>182</v>
-      </c>
-      <c r="B313" t="s">
-        <v>186</v>
+        <v>358</v>
+      </c>
+      <c r="B313">
+        <v>100</v>
+      </c>
+      <c r="C313" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="314" spans="1:3" ht="14.25" customHeight="1">
       <c r="A314" t="s">
-        <v>183</v>
-      </c>
-      <c r="B314" t="s">
-        <v>187</v>
+        <v>361</v>
+      </c>
+      <c r="B314">
+        <v>100</v>
+      </c>
+      <c r="C314" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="315" spans="1:3" ht="14.25" customHeight="1">
       <c r="A315" t="s">
-        <v>185</v>
-      </c>
-      <c r="B315" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="316" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A316" t="s">
-        <v>276</v>
-      </c>
-      <c r="B316" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="317" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="318" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="319" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>364</v>
+      </c>
+      <c r="B315">
+        <v>100</v>
+      </c>
+      <c r="C315" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="317" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A317" t="s">
+        <v>340</v>
+      </c>
+      <c r="B317" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A318" t="s">
+        <v>344</v>
+      </c>
+      <c r="B318" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A319" t="s">
+        <v>347</v>
+      </c>
+      <c r="B319" t="s">
+        <v>348</v>
+      </c>
+    </row>
     <row r="320" spans="1:3" ht="14.25" customHeight="1">
       <c r="A320" t="s">
-        <v>189</v>
-      </c>
-      <c r="B320">
-        <v>5</v>
-      </c>
-      <c r="C320" t="s">
-        <v>48</v>
+        <v>350</v>
+      </c>
+      <c r="B320" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="321" spans="1:3" ht="14.25" customHeight="1">
       <c r="A321" t="s">
-        <v>190</v>
+        <v>353</v>
       </c>
       <c r="B321" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="322" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="323" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="324" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A324" t="s">
-        <v>192</v>
-      </c>
-      <c r="B324">
-        <v>5</v>
-      </c>
-      <c r="C324" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="325" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="326" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="327" spans="1:3" ht="14" customHeight="1">
-      <c r="A327" t="s">
-        <v>344</v>
-      </c>
-      <c r="B327">
-        <v>100</v>
-      </c>
-      <c r="C327" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="328" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A328" t="s">
-        <v>343</v>
-      </c>
-      <c r="B328">
-        <v>100</v>
-      </c>
-      <c r="C328" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="329" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A329" t="s">
-        <v>347</v>
-      </c>
-      <c r="B329">
-        <v>100</v>
-      </c>
-      <c r="C329" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="330" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A330" t="s">
-        <v>350</v>
-      </c>
-      <c r="B330">
-        <v>100</v>
-      </c>
-      <c r="C330" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="331" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A331" t="s">
-        <v>353</v>
-      </c>
-      <c r="B331">
-        <v>100</v>
-      </c>
-      <c r="C331" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="332" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A332" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A322" t="s">
         <v>356</v>
       </c>
-      <c r="B332">
-        <v>100</v>
-      </c>
-      <c r="C332" t="s">
-        <v>72</v>
-      </c>
-    </row>
+      <c r="B322" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A323" t="s">
+        <v>359</v>
+      </c>
+      <c r="B323" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="324" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A324" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="B324" s="6" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="325" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A325" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="B325" s="7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B326" s="7"/>
+    </row>
+    <row r="327" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B327" s="7"/>
+    </row>
+    <row r="328" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="329" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B329" s="7"/>
+    </row>
+    <row r="330" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B330" s="7"/>
+    </row>
+    <row r="331" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B331" s="7"/>
+    </row>
+    <row r="332" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="333" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A333" t="s">
-        <v>359</v>
-      </c>
-      <c r="B333">
-        <v>100</v>
-      </c>
-      <c r="C333" t="s">
-        <v>72</v>
-      </c>
+      <c r="A333" s="6"/>
+      <c r="B333" s="7"/>
+      <c r="C333" s="6"/>
     </row>
     <row r="334" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A334" t="s">
-        <v>362</v>
-      </c>
-      <c r="B334">
-        <v>100</v>
-      </c>
-      <c r="C334" t="s">
-        <v>72</v>
-      </c>
+      <c r="A334" s="6"/>
+      <c r="B334" s="8"/>
+      <c r="C334" s="6"/>
     </row>
     <row r="335" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A335" t="s">
-        <v>365</v>
-      </c>
-      <c r="B335">
-        <v>100</v>
-      </c>
-      <c r="C335" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="336" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="337" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="338" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="339" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="340" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A340" t="s">
-        <v>341</v>
-      </c>
-      <c r="B340" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="341" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A341" t="s">
-        <v>345</v>
-      </c>
-      <c r="B341" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="342" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A342" t="s">
-        <v>348</v>
-      </c>
-      <c r="B342" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="343" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A343" t="s">
-        <v>351</v>
-      </c>
-      <c r="B343" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="344" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A344" t="s">
-        <v>354</v>
-      </c>
-      <c r="B344" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="345" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A345" t="s">
-        <v>357</v>
-      </c>
-      <c r="B345" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="346" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A346" t="s">
-        <v>360</v>
-      </c>
-      <c r="B346" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="347" spans="1:2" s="6" customFormat="1" ht="14.5">
-      <c r="A347" s="6" t="s">
-        <v>363</v>
-      </c>
-      <c r="B347" s="6" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="348" spans="1:2" s="6" customFormat="1" ht="14.5">
-      <c r="A348" s="6" t="s">
-        <v>366</v>
-      </c>
-      <c r="B348" s="7" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="349" spans="1:2" s="6" customFormat="1" ht="14.5">
-      <c r="B349" s="7"/>
-    </row>
-    <row r="350" spans="1:2" s="6" customFormat="1" ht="14.5">
-      <c r="B350" s="7"/>
-    </row>
-    <row r="351" spans="1:2" s="6" customFormat="1" ht="14.5"/>
-    <row r="352" spans="1:2" s="6" customFormat="1" ht="14.5">
-      <c r="B352" s="7"/>
-    </row>
-    <row r="353" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B353" s="7"/>
-    </row>
-    <row r="354" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B354" s="7"/>
-    </row>
-    <row r="355" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="356" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A356" s="6"/>
-      <c r="B356" s="7"/>
-      <c r="C356" s="6"/>
-    </row>
-    <row r="357" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A357" s="6"/>
-      <c r="B357" s="8"/>
-      <c r="C357" s="6"/>
-    </row>
-    <row r="358" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A358" s="6"/>
-      <c r="B358" s="7"/>
-      <c r="C358" s="6"/>
-    </row>
-    <row r="359" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A359" s="6"/>
-      <c r="B359" s="6"/>
-      <c r="C359" s="6"/>
-    </row>
-    <row r="360" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A360" s="6"/>
-      <c r="B360" s="5"/>
-      <c r="C360" s="6"/>
-    </row>
-    <row r="361" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A361" s="6"/>
-      <c r="B361" s="7"/>
-      <c r="C361" s="6"/>
-    </row>
-    <row r="362" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A362" s="6"/>
-      <c r="B362" s="8"/>
-      <c r="C362" s="6"/>
-    </row>
-    <row r="363" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A363" s="6"/>
-      <c r="B363" s="6"/>
-      <c r="C363" s="6"/>
-    </row>
-    <row r="364" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A364" s="6"/>
-      <c r="B364" s="7"/>
-      <c r="C364" s="6"/>
-    </row>
-    <row r="365" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="366" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B366" s="5"/>
-    </row>
-    <row r="367" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B367" s="7"/>
-    </row>
-    <row r="368" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B368" s="8"/>
-    </row>
-    <row r="369" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="370" spans="1:1" ht="14.25" customHeight="1">
-      <c r="A370" s="6"/>
-    </row>
-    <row r="371" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="372" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="373" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="374" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="375" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="376" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="377" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="378" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="379" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="380" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="381" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="382" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="383" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="384" spans="1:1" ht="14.25" customHeight="1"/>
+      <c r="A335" s="6"/>
+      <c r="B335" s="7"/>
+      <c r="C335" s="6"/>
+    </row>
+    <row r="336" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A336" s="6"/>
+      <c r="B336" s="6"/>
+      <c r="C336" s="6"/>
+    </row>
+    <row r="337" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A337" s="6"/>
+      <c r="B337" s="5"/>
+      <c r="C337" s="6"/>
+    </row>
+    <row r="338" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A338" s="6"/>
+      <c r="B338" s="7"/>
+      <c r="C338" s="6"/>
+    </row>
+    <row r="339" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A339" s="6"/>
+      <c r="B339" s="8"/>
+      <c r="C339" s="6"/>
+    </row>
+    <row r="340" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A340" s="6"/>
+      <c r="B340" s="6"/>
+      <c r="C340" s="6"/>
+    </row>
+    <row r="341" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A341" s="6"/>
+      <c r="B341" s="7"/>
+      <c r="C341" s="6"/>
+    </row>
+    <row r="342" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="343" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B343" s="5"/>
+    </row>
+    <row r="344" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B344" s="7"/>
+    </row>
+    <row r="345" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B345" s="8"/>
+    </row>
+    <row r="346" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="347" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A347" s="6"/>
+    </row>
+    <row r="348" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="349" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="350" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="351" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="352" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="353" ht="14.25" customHeight="1"/>
+    <row r="354" ht="14.25" customHeight="1"/>
+    <row r="355" ht="14.25" customHeight="1"/>
+    <row r="356" ht="14.25" customHeight="1"/>
+    <row r="357" ht="14.25" customHeight="1"/>
+    <row r="358" ht="14.25" customHeight="1"/>
+    <row r="359" ht="14.25" customHeight="1"/>
+    <row r="360" ht="14.25" customHeight="1"/>
+    <row r="361" ht="14.25" customHeight="1"/>
+    <row r="362" ht="14.25" customHeight="1"/>
+    <row r="363" ht="14.25" customHeight="1"/>
+    <row r="364" ht="14.25" customHeight="1"/>
+    <row r="365" ht="14.25" customHeight="1"/>
+    <row r="366" ht="14.25" customHeight="1"/>
+    <row r="367" ht="14.25" customHeight="1"/>
+    <row r="368" ht="14.25" customHeight="1"/>
+    <row r="369" ht="14.25" customHeight="1"/>
+    <row r="370" ht="14.25" customHeight="1"/>
+    <row r="371" ht="14.25" customHeight="1"/>
+    <row r="372" ht="14.25" customHeight="1"/>
+    <row r="373" ht="14.25" customHeight="1"/>
+    <row r="374" ht="14.25" customHeight="1"/>
+    <row r="375" ht="14.25" customHeight="1"/>
+    <row r="376" ht="14.25" customHeight="1"/>
+    <row r="377" ht="14.25" customHeight="1"/>
+    <row r="378" ht="14.25" customHeight="1"/>
+    <row r="379" ht="14.25" customHeight="1"/>
+    <row r="380" ht="14.25" customHeight="1"/>
+    <row r="381" ht="14.25" customHeight="1"/>
+    <row r="382" ht="14.25" customHeight="1"/>
+    <row r="383" ht="14.25" customHeight="1"/>
+    <row r="384" ht="14.25" customHeight="1"/>
     <row r="385" ht="14.25" customHeight="1"/>
     <row r="386" ht="14.25" customHeight="1"/>
     <row r="387" ht="14.25" customHeight="1"/>
@@ -5359,29 +5373,6 @@
     <row r="1201" ht="14.25" customHeight="1"/>
     <row r="1202" ht="14.25" customHeight="1"/>
     <row r="1203" ht="14.25" customHeight="1"/>
-    <row r="1204" ht="14.25" customHeight="1"/>
-    <row r="1205" ht="14.25" customHeight="1"/>
-    <row r="1206" ht="14.25" customHeight="1"/>
-    <row r="1207" ht="14.25" customHeight="1"/>
-    <row r="1208" ht="14.25" customHeight="1"/>
-    <row r="1209" ht="14.25" customHeight="1"/>
-    <row r="1210" ht="14.25" customHeight="1"/>
-    <row r="1211" ht="14.25" customHeight="1"/>
-    <row r="1212" ht="14.25" customHeight="1"/>
-    <row r="1213" ht="14.25" customHeight="1"/>
-    <row r="1214" ht="14.25" customHeight="1"/>
-    <row r="1215" ht="14.25" customHeight="1"/>
-    <row r="1216" ht="14.25" customHeight="1"/>
-    <row r="1217" ht="14.25" customHeight="1"/>
-    <row r="1218" ht="14.25" customHeight="1"/>
-    <row r="1219" ht="14.25" customHeight="1"/>
-    <row r="1220" ht="14.25" customHeight="1"/>
-    <row r="1221" ht="14.25" customHeight="1"/>
-    <row r="1222" ht="14.25" customHeight="1"/>
-    <row r="1223" ht="14.25" customHeight="1"/>
-    <row r="1224" ht="14.25" customHeight="1"/>
-    <row r="1225" ht="14.25" customHeight="1"/>
-    <row r="1226" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5576,7 +5567,7 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1"/>

</xml_diff>